<commit_message>
adding teacher data from excel (update)
</commit_message>
<xml_diff>
--- a/bin/excel_resources/excel_data.xlsx
+++ b/bin/excel_resources/excel_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0096F69B-4092-4F6A-8C5A-42D95CF2F431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC5D553-17FE-4946-B674-2E2A9B8E2F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="72">
   <si>
     <t>10A1</t>
   </si>
@@ -140,9 +140,6 @@
   </si>
   <si>
     <t>Tự Nhiên</t>
-  </si>
-  <si>
-    <t>Ban Giáo Hiệu</t>
   </si>
   <si>
     <t>Tên môn học</t>
@@ -282,7 +279,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -388,6 +385,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -407,13 +413,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -428,19 +436,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -748,8 +756,8 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="18" t="s">
-        <v>72</v>
+      <c r="A5" s="9" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -772,15 +780,15 @@
         <v>33</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="C7" s="1" t="str">
         <f>A47</f>
@@ -800,7 +808,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>12</v>
@@ -921,8 +929,8 @@
       <c r="G19" s="1"/>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A21" s="18" t="s">
-        <v>68</v>
+      <c r="A21" s="9" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.35">
@@ -934,26 +942,26 @@
       <c r="A23" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-      <c r="T23" s="13"/>
-      <c r="U23" s="13"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
@@ -986,104 +994,104 @@
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" s="17" t="s">
+      <c r="A38" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="17" t="s">
+      <c r="A39" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="17" t="s">
+      <c r="A41" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" s="19" t="s">
-        <v>69</v>
+      <c r="A44" s="10" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="C45" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="F45" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" s="2">
         <v>1</v>
       </c>
       <c r="C46" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" ref="C46:C62" si="0">A$81</f>
         <v>Sáng</v>
       </c>
       <c r="D46" s="2">
@@ -1100,13 +1108,13 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="2">
         <v>1</v>
       </c>
       <c r="C47" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D47" s="2">
@@ -1123,13 +1131,13 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B48" s="2">
         <v>1</v>
       </c>
       <c r="C48" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D48" s="2">
@@ -1146,188 +1154,182 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B49" s="2">
         <v>1</v>
       </c>
       <c r="C49" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D49" s="2">
         <v>1</v>
       </c>
       <c r="E49" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" ref="E49:E62" si="1">B$82</f>
         <v>0</v>
       </c>
       <c r="F49" s="2" t="str">
         <f>A$66</f>
         <v>Xã Hội</v>
       </c>
-      <c r="G49" s="13"/>
+      <c r="G49" s="6"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B50" s="2">
         <v>1</v>
       </c>
       <c r="C50" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D50" s="2">
         <v>1</v>
       </c>
       <c r="E50" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F50" s="2" t="str">
         <f>A$66</f>
         <v>Xã Hội</v>
       </c>
-      <c r="G50" s="14"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B51" s="2">
         <v>1</v>
       </c>
       <c r="C51" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D51" s="2">
         <v>1</v>
       </c>
       <c r="E51" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F51" s="2" t="str">
         <f>A$67</f>
         <v>Tự Nhiên</v>
       </c>
-      <c r="G51" s="14"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B52" s="2">
         <v>1</v>
       </c>
       <c r="C52" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D52" s="2">
         <v>1</v>
       </c>
       <c r="E52" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F52" s="2" t="str">
         <f>A$67</f>
         <v>Tự Nhiên</v>
       </c>
-      <c r="G52" s="14"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B53" s="2">
         <v>1</v>
       </c>
       <c r="C53" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D53" s="2">
         <v>1</v>
       </c>
       <c r="E53" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F53" s="2" t="str">
         <f>A$67</f>
         <v>Tự Nhiên</v>
       </c>
-      <c r="G53" s="14"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B54" s="2">
         <v>2</v>
       </c>
       <c r="C54" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D54" s="2">
         <v>2</v>
       </c>
       <c r="E54" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F54" s="2" t="str">
         <f>A$67</f>
         <v>Tự Nhiên</v>
       </c>
-      <c r="G54" s="14"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B55" s="2">
         <v>2</v>
       </c>
       <c r="C55" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D55" s="2">
         <v>2</v>
       </c>
       <c r="E55" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F55" s="2" t="str">
         <f>A$66</f>
         <v>Xã Hội</v>
       </c>
-      <c r="G55" s="14"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B56" s="2">
         <v>1</v>
       </c>
       <c r="C56" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D56" s="2">
         <v>1</v>
       </c>
       <c r="E56" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F56" s="2" t="str">
@@ -1337,20 +1339,20 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B57" s="2">
         <v>2</v>
       </c>
       <c r="C57" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D57" s="2">
         <v>2</v>
       </c>
       <c r="E57" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F57" s="2" t="str">
@@ -1360,20 +1362,20 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B58" s="2">
         <v>2</v>
       </c>
       <c r="C58" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D58" s="2">
         <v>2</v>
       </c>
       <c r="E58" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F58" s="2" t="str">
@@ -1383,20 +1385,20 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B59" s="2">
         <v>2</v>
       </c>
       <c r="C59" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D59" s="2">
         <v>2</v>
       </c>
       <c r="E59" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F59" s="2" t="str">
@@ -1406,20 +1408,20 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B60" s="2">
         <v>2</v>
       </c>
       <c r="C60" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D60" s="2">
         <v>2</v>
       </c>
       <c r="E60" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F60" s="2" t="str">
@@ -1429,20 +1431,20 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B61" s="2">
         <v>1</v>
       </c>
       <c r="C61" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D61" s="2">
         <v>1</v>
       </c>
       <c r="E61" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F61" s="2" t="str">
@@ -1452,20 +1454,20 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B62" s="2">
         <v>1</v>
       </c>
       <c r="C62" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D62" s="2">
         <v>1</v>
       </c>
       <c r="E62" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F62" s="2" t="str">
@@ -1474,17 +1476,17 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A64" s="18" t="s">
-        <v>70</v>
+      <c r="A64" s="9" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B65" s="15"/>
-      <c r="C65" s="13"/>
-      <c r="D65" s="13"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="6"/>
+      <c r="D65" s="6"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
@@ -1492,108 +1494,79 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67" s="2" t="s">
+      <c r="A67" s="18" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A68" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C68" s="13"/>
-      <c r="D68" s="13"/>
-      <c r="E68" s="13"/>
-      <c r="F68" s="13"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C69" s="14"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="14"/>
-      <c r="F69" s="14"/>
+      <c r="A68" s="19"/>
+      <c r="C68" s="6"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="6"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="C70" s="14"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="14"/>
-      <c r="F70" s="14"/>
+      <c r="A70" s="10" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B71" s="15"/>
-      <c r="C71" s="14"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="14"/>
-      <c r="F71" s="14"/>
+        <v>64</v>
+      </c>
+      <c r="B71" s="7"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B72" s="16"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
+      <c r="B72" s="8"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B73" s="16"/>
-      <c r="C73" s="14"/>
-      <c r="D73" s="14"/>
-      <c r="E73" s="14"/>
-      <c r="F73" s="14"/>
+      <c r="B73" s="8"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B74" s="16"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
+      <c r="B74" s="8"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B75" s="16"/>
+      <c r="B75" s="8"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B76" s="16"/>
+      <c r="B76" s="8"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B77" s="16"/>
-      <c r="C77" s="13"/>
+      <c r="B77" s="8"/>
+      <c r="C77" s="6"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C78" s="13"/>
+      <c r="C78" s="6"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A79" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="C79" s="14"/>
+      <c r="A79" s="9" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.35">
@@ -1606,7 +1579,7 @@
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A82" s="17" t="s">
+      <c r="A82" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B82" s="1" t="b">
@@ -1626,28 +1599,28 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
-      <c r="T4" s="7"/>
-      <c r="U4" s="7"/>
-      <c r="V4" s="8"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="16"/>
+      <c r="S4" s="16"/>
+      <c r="T4" s="16"/>
+      <c r="U4" s="16"/>
+      <c r="V4" s="17"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -1713,7 +1686,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -1741,7 +1714,7 @@
       <c r="V6" s="1"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="9"/>
+      <c r="A7" s="11"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -1767,7 +1740,7 @@
       <c r="V7" s="1"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="9"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -1793,7 +1766,7 @@
       <c r="V8" s="1"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="9"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -1819,7 +1792,7 @@
       <c r="V9" s="1"/>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="9"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -1845,7 +1818,7 @@
       <c r="V10" s="1"/>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -1873,7 +1846,7 @@
       <c r="V11" s="1"/>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="11"/>
+      <c r="A12" s="13"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -1899,7 +1872,7 @@
       <c r="V12" s="1"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="12"/>
+      <c r="A13" s="14"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -1925,28 +1898,28 @@
       <c r="V13" s="1"/>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="7"/>
-      <c r="S16" s="7"/>
-      <c r="T16" s="7"/>
-      <c r="U16" s="7"/>
-      <c r="V16" s="8"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="16"/>
+      <c r="T16" s="16"/>
+      <c r="U16" s="16"/>
+      <c r="V16" s="17"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -2012,7 +1985,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
@@ -2040,7 +2013,7 @@
       <c r="V18" s="1"/>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="9"/>
+      <c r="A19" s="11"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -2066,7 +2039,7 @@
       <c r="V19" s="1"/>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="9"/>
+      <c r="A20" s="11"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -2092,7 +2065,7 @@
       <c r="V20" s="1"/>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="9"/>
+      <c r="A21" s="11"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -2118,7 +2091,7 @@
       <c r="V21" s="1"/>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="9"/>
+      <c r="A22" s="11"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -2144,7 +2117,7 @@
       <c r="V22" s="1"/>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -2172,7 +2145,7 @@
       <c r="V23" s="1"/>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="11"/>
+      <c r="A24" s="13"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -2198,7 +2171,7 @@
       <c r="V24" s="1"/>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="12"/>
+      <c r="A25" s="14"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -2224,28 +2197,28 @@
       <c r="V25" s="1"/>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
-      <c r="N28" s="7"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="7"/>
-      <c r="R28" s="7"/>
-      <c r="S28" s="7"/>
-      <c r="T28" s="7"/>
-      <c r="U28" s="7"/>
-      <c r="V28" s="8"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="16"/>
+      <c r="T28" s="16"/>
+      <c r="U28" s="16"/>
+      <c r="V28" s="17"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -2311,7 +2284,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -2339,7 +2312,7 @@
       <c r="V30" s="1"/>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="9"/>
+      <c r="A31" s="11"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -2365,7 +2338,7 @@
       <c r="V31" s="1"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="9"/>
+      <c r="A32" s="11"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -2391,7 +2364,7 @@
       <c r="V32" s="1"/>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="9"/>
+      <c r="A33" s="11"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -2417,7 +2390,7 @@
       <c r="V33" s="1"/>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="9"/>
+      <c r="A34" s="11"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -2443,7 +2416,7 @@
       <c r="V34" s="1"/>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -2471,7 +2444,7 @@
       <c r="V35" s="1"/>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="11"/>
+      <c r="A36" s="13"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -2497,7 +2470,7 @@
       <c r="V36" s="1"/>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="12"/>
+      <c r="A37" s="14"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -2523,28 +2496,28 @@
       <c r="V37" s="1"/>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="7"/>
-      <c r="J40" s="7"/>
-      <c r="K40" s="7"/>
-      <c r="L40" s="7"/>
-      <c r="M40" s="7"/>
-      <c r="N40" s="7"/>
-      <c r="O40" s="7"/>
-      <c r="P40" s="7"/>
-      <c r="Q40" s="7"/>
-      <c r="R40" s="7"/>
-      <c r="S40" s="7"/>
-      <c r="T40" s="7"/>
-      <c r="U40" s="7"/>
-      <c r="V40" s="8"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
+      <c r="L40" s="16"/>
+      <c r="M40" s="16"/>
+      <c r="N40" s="16"/>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="Q40" s="16"/>
+      <c r="R40" s="16"/>
+      <c r="S40" s="16"/>
+      <c r="T40" s="16"/>
+      <c r="U40" s="16"/>
+      <c r="V40" s="17"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -2610,7 +2583,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -2638,7 +2611,7 @@
       <c r="V42" s="1"/>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="9"/>
+      <c r="A43" s="11"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -2664,7 +2637,7 @@
       <c r="V43" s="1"/>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="9"/>
+      <c r="A44" s="11"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -2690,7 +2663,7 @@
       <c r="V44" s="1"/>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="9"/>
+      <c r="A45" s="11"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -2716,7 +2689,7 @@
       <c r="V45" s="1"/>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="9"/>
+      <c r="A46" s="11"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -2742,7 +2715,7 @@
       <c r="V46" s="1"/>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -2770,7 +2743,7 @@
       <c r="V47" s="1"/>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="11"/>
+      <c r="A48" s="13"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -2796,7 +2769,7 @@
       <c r="V48" s="1"/>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="12"/>
+      <c r="A49" s="14"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -2822,28 +2795,28 @@
       <c r="V49" s="1"/>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="7"/>
-      <c r="E52" s="7"/>
-      <c r="F52" s="7"/>
-      <c r="G52" s="7"/>
-      <c r="H52" s="7"/>
-      <c r="I52" s="7"/>
-      <c r="J52" s="7"/>
-      <c r="K52" s="7"/>
-      <c r="L52" s="7"/>
-      <c r="M52" s="7"/>
-      <c r="N52" s="7"/>
-      <c r="O52" s="7"/>
-      <c r="P52" s="7"/>
-      <c r="Q52" s="7"/>
-      <c r="R52" s="7"/>
-      <c r="S52" s="7"/>
-      <c r="T52" s="7"/>
-      <c r="U52" s="7"/>
-      <c r="V52" s="8"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="16"/>
+      <c r="L52" s="16"/>
+      <c r="M52" s="16"/>
+      <c r="N52" s="16"/>
+      <c r="O52" s="16"/>
+      <c r="P52" s="16"/>
+      <c r="Q52" s="16"/>
+      <c r="R52" s="16"/>
+      <c r="S52" s="16"/>
+      <c r="T52" s="16"/>
+      <c r="U52" s="16"/>
+      <c r="V52" s="17"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -2909,7 +2882,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="9" t="s">
+      <c r="A54" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
@@ -2937,7 +2910,7 @@
       <c r="V54" s="1"/>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="9"/>
+      <c r="A55" s="11"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -2963,7 +2936,7 @@
       <c r="V55" s="1"/>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="9"/>
+      <c r="A56" s="11"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -2989,7 +2962,7 @@
       <c r="V56" s="1"/>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="9"/>
+      <c r="A57" s="11"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -3015,7 +2988,7 @@
       <c r="V57" s="1"/>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="9"/>
+      <c r="A58" s="11"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -3041,7 +3014,7 @@
       <c r="V58" s="1"/>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="10" t="s">
+      <c r="A59" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -3069,7 +3042,7 @@
       <c r="V59" s="1"/>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="11"/>
+      <c r="A60" s="13"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -3095,7 +3068,7 @@
       <c r="V60" s="1"/>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="12"/>
+      <c r="A61" s="14"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -3121,28 +3094,28 @@
       <c r="V61" s="1"/>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="6" t="s">
+      <c r="C64" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="7"/>
-      <c r="E64" s="7"/>
-      <c r="F64" s="7"/>
-      <c r="G64" s="7"/>
-      <c r="H64" s="7"/>
-      <c r="I64" s="7"/>
-      <c r="J64" s="7"/>
-      <c r="K64" s="7"/>
-      <c r="L64" s="7"/>
-      <c r="M64" s="7"/>
-      <c r="N64" s="7"/>
-      <c r="O64" s="7"/>
-      <c r="P64" s="7"/>
-      <c r="Q64" s="7"/>
-      <c r="R64" s="7"/>
-      <c r="S64" s="7"/>
-      <c r="T64" s="7"/>
-      <c r="U64" s="7"/>
-      <c r="V64" s="8"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+      <c r="G64" s="16"/>
+      <c r="H64" s="16"/>
+      <c r="I64" s="16"/>
+      <c r="J64" s="16"/>
+      <c r="K64" s="16"/>
+      <c r="L64" s="16"/>
+      <c r="M64" s="16"/>
+      <c r="N64" s="16"/>
+      <c r="O64" s="16"/>
+      <c r="P64" s="16"/>
+      <c r="Q64" s="16"/>
+      <c r="R64" s="16"/>
+      <c r="S64" s="16"/>
+      <c r="T64" s="16"/>
+      <c r="U64" s="16"/>
+      <c r="V64" s="17"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -3208,7 +3181,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="9" t="s">
+      <c r="A66" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -3236,7 +3209,7 @@
       <c r="V66" s="1"/>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="9"/>
+      <c r="A67" s="11"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -3262,7 +3235,7 @@
       <c r="V67" s="1"/>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="9"/>
+      <c r="A68" s="11"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -3288,7 +3261,7 @@
       <c r="V68" s="1"/>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="9"/>
+      <c r="A69" s="11"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -3314,7 +3287,7 @@
       <c r="V69" s="1"/>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="9"/>
+      <c r="A70" s="11"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -3340,7 +3313,7 @@
       <c r="V70" s="1"/>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="10" t="s">
+      <c r="A71" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -3368,7 +3341,7 @@
       <c r="V71" s="1"/>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="11"/>
+      <c r="A72" s="13"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -3394,7 +3367,7 @@
       <c r="V72" s="1"/>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="12"/>
+      <c r="A73" s="14"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -3421,6 +3394,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -3429,16 +3412,6 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
display data into excel
</commit_message>
<xml_diff>
--- a/bin/excel_resources/excel_data.xlsx
+++ b/bin/excel_resources/excel_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC5D553-17FE-4946-B674-2E2A9B8E2F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E76DB2-2EA3-4178-9C49-E9834DB93D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="73">
   <si>
     <t>10A1</t>
   </si>
@@ -242,6 +242,9 @@
   </si>
   <si>
     <t>Giáo Viên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tổ </t>
   </si>
 </sst>
 </file>
@@ -424,6 +427,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -435,21 +453,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -755,12 +758,12 @@
     <col min="21" max="21" width="9.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -779,11 +782,14 @@
       <c r="F6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H6" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>65</v>
       </c>
@@ -805,8 +811,12 @@
         <f>A75</f>
         <v>Thứ Năm</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H7" s="1" t="str">
+        <f>F$47</f>
+        <v>Xã Hội</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>65</v>
       </c>
@@ -828,8 +838,12 @@
         <f>A75</f>
         <v>Thứ Năm</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H8" s="1" t="str">
+        <f>F$47</f>
+        <v>Xã Hội</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -837,8 +851,9 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -846,8 +861,9 @@
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H10" s="1"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -855,8 +871,9 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -864,8 +881,9 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H12" s="1"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -873,8 +891,9 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -882,8 +901,9 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -891,8 +911,9 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -900,6 +921,7 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
@@ -909,6 +931,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
@@ -918,6 +941,7 @@
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
@@ -927,6 +951,7 @@
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
@@ -1494,12 +1519,12 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67" s="18" t="s">
+      <c r="A67" s="11" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A68" s="19"/>
+      <c r="A68" s="12"/>
       <c r="C68" s="6"/>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
@@ -1599,28 +1624,28 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="16"/>
-      <c r="U4" s="16"/>
-      <c r="V4" s="17"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="14"/>
+      <c r="S4" s="14"/>
+      <c r="T4" s="14"/>
+      <c r="U4" s="14"/>
+      <c r="V4" s="15"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -1686,7 +1711,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -1714,7 +1739,7 @@
       <c r="V6" s="1"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="11"/>
+      <c r="A7" s="16"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -1740,7 +1765,7 @@
       <c r="V7" s="1"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="11"/>
+      <c r="A8" s="16"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -1766,7 +1791,7 @@
       <c r="V8" s="1"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="11"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -1792,7 +1817,7 @@
       <c r="V9" s="1"/>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="11"/>
+      <c r="A10" s="16"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -1818,7 +1843,7 @@
       <c r="V10" s="1"/>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -1846,7 +1871,7 @@
       <c r="V11" s="1"/>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="13"/>
+      <c r="A12" s="18"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -1872,7 +1897,7 @@
       <c r="V12" s="1"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="14"/>
+      <c r="A13" s="19"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -1898,28 +1923,28 @@
       <c r="V13" s="1"/>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="16"/>
-      <c r="O16" s="16"/>
-      <c r="P16" s="16"/>
-      <c r="Q16" s="16"/>
-      <c r="R16" s="16"/>
-      <c r="S16" s="16"/>
-      <c r="T16" s="16"/>
-      <c r="U16" s="16"/>
-      <c r="V16" s="17"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="14"/>
+      <c r="S16" s="14"/>
+      <c r="T16" s="14"/>
+      <c r="U16" s="14"/>
+      <c r="V16" s="15"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -1985,7 +2010,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
@@ -2013,7 +2038,7 @@
       <c r="V18" s="1"/>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="11"/>
+      <c r="A19" s="16"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -2039,7 +2064,7 @@
       <c r="V19" s="1"/>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="11"/>
+      <c r="A20" s="16"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -2065,7 +2090,7 @@
       <c r="V20" s="1"/>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="11"/>
+      <c r="A21" s="16"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -2091,7 +2116,7 @@
       <c r="V21" s="1"/>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="11"/>
+      <c r="A22" s="16"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -2117,7 +2142,7 @@
       <c r="V22" s="1"/>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -2145,7 +2170,7 @@
       <c r="V23" s="1"/>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="13"/>
+      <c r="A24" s="18"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -2171,7 +2196,7 @@
       <c r="V24" s="1"/>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="14"/>
+      <c r="A25" s="19"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -2197,28 +2222,28 @@
       <c r="V25" s="1"/>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="16"/>
-      <c r="O28" s="16"/>
-      <c r="P28" s="16"/>
-      <c r="Q28" s="16"/>
-      <c r="R28" s="16"/>
-      <c r="S28" s="16"/>
-      <c r="T28" s="16"/>
-      <c r="U28" s="16"/>
-      <c r="V28" s="17"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+      <c r="M28" s="14"/>
+      <c r="N28" s="14"/>
+      <c r="O28" s="14"/>
+      <c r="P28" s="14"/>
+      <c r="Q28" s="14"/>
+      <c r="R28" s="14"/>
+      <c r="S28" s="14"/>
+      <c r="T28" s="14"/>
+      <c r="U28" s="14"/>
+      <c r="V28" s="15"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -2284,7 +2309,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -2312,7 +2337,7 @@
       <c r="V30" s="1"/>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="11"/>
+      <c r="A31" s="16"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -2338,7 +2363,7 @@
       <c r="V31" s="1"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="11"/>
+      <c r="A32" s="16"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -2364,7 +2389,7 @@
       <c r="V32" s="1"/>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="11"/>
+      <c r="A33" s="16"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -2390,7 +2415,7 @@
       <c r="V33" s="1"/>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="11"/>
+      <c r="A34" s="16"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -2416,7 +2441,7 @@
       <c r="V34" s="1"/>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -2444,7 +2469,7 @@
       <c r="V35" s="1"/>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="13"/>
+      <c r="A36" s="18"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -2470,7 +2495,7 @@
       <c r="V36" s="1"/>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="14"/>
+      <c r="A37" s="19"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -2496,28 +2521,28 @@
       <c r="V37" s="1"/>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="15" t="s">
+      <c r="C40" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
-      <c r="G40" s="16"/>
-      <c r="H40" s="16"/>
-      <c r="I40" s="16"/>
-      <c r="J40" s="16"/>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="16"/>
-      <c r="O40" s="16"/>
-      <c r="P40" s="16"/>
-      <c r="Q40" s="16"/>
-      <c r="R40" s="16"/>
-      <c r="S40" s="16"/>
-      <c r="T40" s="16"/>
-      <c r="U40" s="16"/>
-      <c r="V40" s="17"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="14"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="14"/>
+      <c r="L40" s="14"/>
+      <c r="M40" s="14"/>
+      <c r="N40" s="14"/>
+      <c r="O40" s="14"/>
+      <c r="P40" s="14"/>
+      <c r="Q40" s="14"/>
+      <c r="R40" s="14"/>
+      <c r="S40" s="14"/>
+      <c r="T40" s="14"/>
+      <c r="U40" s="14"/>
+      <c r="V40" s="15"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -2583,7 +2608,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="11" t="s">
+      <c r="A42" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -2611,7 +2636,7 @@
       <c r="V42" s="1"/>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="11"/>
+      <c r="A43" s="16"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -2637,7 +2662,7 @@
       <c r="V43" s="1"/>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="11"/>
+      <c r="A44" s="16"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -2663,7 +2688,7 @@
       <c r="V44" s="1"/>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="11"/>
+      <c r="A45" s="16"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -2689,7 +2714,7 @@
       <c r="V45" s="1"/>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="11"/>
+      <c r="A46" s="16"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -2715,7 +2740,7 @@
       <c r="V46" s="1"/>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="12" t="s">
+      <c r="A47" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -2743,7 +2768,7 @@
       <c r="V47" s="1"/>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="13"/>
+      <c r="A48" s="18"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -2769,7 +2794,7 @@
       <c r="V48" s="1"/>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="14"/>
+      <c r="A49" s="19"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -2795,28 +2820,28 @@
       <c r="V49" s="1"/>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="15" t="s">
+      <c r="C52" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="16"/>
-      <c r="E52" s="16"/>
-      <c r="F52" s="16"/>
-      <c r="G52" s="16"/>
-      <c r="H52" s="16"/>
-      <c r="I52" s="16"/>
-      <c r="J52" s="16"/>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="16"/>
-      <c r="O52" s="16"/>
-      <c r="P52" s="16"/>
-      <c r="Q52" s="16"/>
-      <c r="R52" s="16"/>
-      <c r="S52" s="16"/>
-      <c r="T52" s="16"/>
-      <c r="U52" s="16"/>
-      <c r="V52" s="17"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
+      <c r="H52" s="14"/>
+      <c r="I52" s="14"/>
+      <c r="J52" s="14"/>
+      <c r="K52" s="14"/>
+      <c r="L52" s="14"/>
+      <c r="M52" s="14"/>
+      <c r="N52" s="14"/>
+      <c r="O52" s="14"/>
+      <c r="P52" s="14"/>
+      <c r="Q52" s="14"/>
+      <c r="R52" s="14"/>
+      <c r="S52" s="14"/>
+      <c r="T52" s="14"/>
+      <c r="U52" s="14"/>
+      <c r="V52" s="15"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -2882,7 +2907,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="11" t="s">
+      <c r="A54" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
@@ -2910,7 +2935,7 @@
       <c r="V54" s="1"/>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="11"/>
+      <c r="A55" s="16"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -2936,7 +2961,7 @@
       <c r="V55" s="1"/>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="11"/>
+      <c r="A56" s="16"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -2962,7 +2987,7 @@
       <c r="V56" s="1"/>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="11"/>
+      <c r="A57" s="16"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -2988,7 +3013,7 @@
       <c r="V57" s="1"/>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="11"/>
+      <c r="A58" s="16"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -3014,7 +3039,7 @@
       <c r="V58" s="1"/>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -3042,7 +3067,7 @@
       <c r="V59" s="1"/>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="13"/>
+      <c r="A60" s="18"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -3068,7 +3093,7 @@
       <c r="V60" s="1"/>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="14"/>
+      <c r="A61" s="19"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -3094,28 +3119,28 @@
       <c r="V61" s="1"/>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="15" t="s">
+      <c r="C64" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="16"/>
-      <c r="E64" s="16"/>
-      <c r="F64" s="16"/>
-      <c r="G64" s="16"/>
-      <c r="H64" s="16"/>
-      <c r="I64" s="16"/>
-      <c r="J64" s="16"/>
-      <c r="K64" s="16"/>
-      <c r="L64" s="16"/>
-      <c r="M64" s="16"/>
-      <c r="N64" s="16"/>
-      <c r="O64" s="16"/>
-      <c r="P64" s="16"/>
-      <c r="Q64" s="16"/>
-      <c r="R64" s="16"/>
-      <c r="S64" s="16"/>
-      <c r="T64" s="16"/>
-      <c r="U64" s="16"/>
-      <c r="V64" s="17"/>
+      <c r="D64" s="14"/>
+      <c r="E64" s="14"/>
+      <c r="F64" s="14"/>
+      <c r="G64" s="14"/>
+      <c r="H64" s="14"/>
+      <c r="I64" s="14"/>
+      <c r="J64" s="14"/>
+      <c r="K64" s="14"/>
+      <c r="L64" s="14"/>
+      <c r="M64" s="14"/>
+      <c r="N64" s="14"/>
+      <c r="O64" s="14"/>
+      <c r="P64" s="14"/>
+      <c r="Q64" s="14"/>
+      <c r="R64" s="14"/>
+      <c r="S64" s="14"/>
+      <c r="T64" s="14"/>
+      <c r="U64" s="14"/>
+      <c r="V64" s="15"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -3181,7 +3206,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="11" t="s">
+      <c r="A66" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -3209,7 +3234,7 @@
       <c r="V66" s="1"/>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="11"/>
+      <c r="A67" s="16"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -3235,7 +3260,7 @@
       <c r="V67" s="1"/>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="11"/>
+      <c r="A68" s="16"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -3261,7 +3286,7 @@
       <c r="V68" s="1"/>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="11"/>
+      <c r="A69" s="16"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -3287,7 +3312,7 @@
       <c r="V69" s="1"/>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="11"/>
+      <c r="A70" s="16"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -3313,7 +3338,7 @@
       <c r="V70" s="1"/>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="12" t="s">
+      <c r="A71" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -3341,7 +3366,7 @@
       <c r="V71" s="1"/>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="13"/>
+      <c r="A72" s="18"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -3367,7 +3392,7 @@
       <c r="V72" s="1"/>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="14"/>
+      <c r="A73" s="19"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -3394,16 +3419,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -3412,6 +3427,16 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
priotize arrange essential course first
</commit_message>
<xml_diff>
--- a/bin/excel_resources/excel_data.xlsx
+++ b/bin/excel_resources/excel_data.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E688D8-8030-470B-89B1-B8AA50223940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA6B1EB5-25AE-4BB2-9D19-D0E02F79F37E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5052" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="107">
   <si>
     <t>10A1</t>
   </si>
@@ -310,13 +310,7 @@
     <t>Hoàng Văn Chinh-CD Sử</t>
   </si>
   <si>
-    <t>Cao Thị Tố Uyên-CD Văn</t>
-  </si>
-  <si>
     <t>Hoàng Hiếu Trình-CD Văn</t>
-  </si>
-  <si>
-    <t>Nguyễn Thị Hằng-CD Sử</t>
   </si>
   <si>
     <t>1,2</t>
@@ -359,7 +353,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -510,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -555,6 +548,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -566,18 +568,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -862,25 +852,25 @@
   <dimension ref="A5:U124"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="28.08984375"/>
-    <col min="2" max="2" customWidth="true" width="63.08984375"/>
-    <col min="3" max="3" customWidth="true" width="20.1796875"/>
-    <col min="4" max="4" customWidth="true" width="16.36328125"/>
-    <col min="5" max="5" customWidth="true" width="15.26953125"/>
-    <col min="6" max="6" customWidth="true" width="22.7265625"/>
-    <col min="7" max="7" customWidth="true" width="21.54296875"/>
-    <col min="8" max="8" customWidth="true" width="20.36328125"/>
-    <col min="9" max="9" customWidth="true" width="26.453125"/>
-    <col min="10" max="10" customWidth="true" width="22.81640625"/>
-    <col min="11" max="11" customWidth="true" width="23.36328125"/>
-    <col min="12" max="12" customWidth="true" width="12.7265625"/>
-    <col min="13" max="13" customWidth="true" width="19.1796875"/>
-    <col min="14" max="14" customWidth="true" width="16.08984375"/>
-    <col min="15" max="15" customWidth="true" width="16.1796875"/>
-    <col min="16" max="16" customWidth="true" width="10.90625"/>
-    <col min="17" max="17" customWidth="true" width="13.54296875"/>
-    <col min="20" max="20" customWidth="true" width="17.08984375"/>
-    <col min="21" max="21" customWidth="true" width="9.90625"/>
+    <col min="1" max="1" width="28.08984375" customWidth="1"/>
+    <col min="2" max="2" width="63.08984375" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" customWidth="1"/>
+    <col min="6" max="6" width="22.7265625" customWidth="1"/>
+    <col min="7" max="7" width="21.54296875" customWidth="1"/>
+    <col min="8" max="8" width="20.36328125" customWidth="1"/>
+    <col min="9" max="9" width="26.453125" customWidth="1"/>
+    <col min="10" max="10" width="22.81640625" customWidth="1"/>
+    <col min="11" max="11" width="23.36328125" customWidth="1"/>
+    <col min="12" max="12" width="12.7265625" customWidth="1"/>
+    <col min="13" max="13" width="19.1796875" customWidth="1"/>
+    <col min="14" max="14" width="16.08984375" customWidth="1"/>
+    <col min="15" max="15" width="16.1796875" customWidth="1"/>
+    <col min="16" max="16" width="10.90625" customWidth="1"/>
+    <col min="17" max="17" width="13.54296875" customWidth="1"/>
+    <col min="20" max="20" width="17.08984375" customWidth="1"/>
+    <col min="21" max="21" width="9.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -905,22 +895,22 @@
         <v>32</v>
       </c>
       <c r="F6" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="H6" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="I6" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="H6" s="16" t="s">
+      <c r="J6" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="I6" s="25" t="s">
+      <c r="K6" s="16" t="s">
         <v>102</v>
-      </c>
-      <c r="J6" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="K6" s="16" t="s">
-        <v>104</v>
       </c>
       <c r="L6" s="14" t="s">
         <v>62</v>
@@ -946,28 +936,18 @@
       <c r="E7" s="13">
         <v>105</v>
       </c>
-      <c r="F7" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>105</v>
-      </c>
+      <c r="F7" s="13"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>98</v>
-      </c>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
       <c r="L7" s="13" t="str">
         <f>A117</f>
         <v>Thứ Năm</v>
       </c>
       <c r="M7" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" ref="M7:M18" si="0">F$89</f>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -989,27 +969,27 @@
         <v>35</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L8" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" ref="L8:L18" si="1">A$117</f>
         <v>Thứ Năm</v>
       </c>
       <c r="M8" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1030,18 +1010,28 @@
       <c r="E9" s="13">
         <v>105</v>
       </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
+      <c r="F9" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>96</v>
+      </c>
       <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="J9" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>95</v>
+      </c>
       <c r="L9" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M9" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1068,11 +1058,11 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M10" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1100,11 +1090,11 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M11" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1131,11 +1121,11 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M12" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1163,11 +1153,11 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M13" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1194,11 +1184,11 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M14" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1226,11 +1216,11 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
       <c r="L15" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M15" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1258,11 +1248,11 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
       <c r="L16" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M16" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1290,11 +1280,11 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M17" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1322,11 +1312,11 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="13" t="str">
-        <f>A$117</f>
+        <f t="shared" si="1"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M18" s="13" t="str">
-        <f>F$89</f>
+        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1669,7 +1659,7 @@
         <v>1</v>
       </c>
       <c r="C88" s="2" t="str">
-        <f t="shared" ref="C88:C104" si="0">A$123</f>
+        <f t="shared" ref="C88:C104" si="2">A$123</f>
         <v>Sáng</v>
       </c>
       <c r="D88" s="2">
@@ -1692,7 +1682,7 @@
         <v>1</v>
       </c>
       <c r="C89" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D89" s="2">
@@ -1715,7 +1705,7 @@
         <v>1</v>
       </c>
       <c r="C90" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D90" s="2">
@@ -1738,14 +1728,14 @@
         <v>1</v>
       </c>
       <c r="C91" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D91" s="2">
         <v>1</v>
       </c>
       <c r="E91" s="2" t="b">
-        <f t="shared" ref="E91:E104" si="1">B$124</f>
+        <f t="shared" ref="E91:E104" si="3">B$124</f>
         <v>0</v>
       </c>
       <c r="F91" s="2" t="str">
@@ -1762,14 +1752,14 @@
         <v>1</v>
       </c>
       <c r="C92" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D92" s="2">
         <v>1</v>
       </c>
       <c r="E92" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F92" s="2" t="str">
@@ -1785,14 +1775,14 @@
         <v>1</v>
       </c>
       <c r="C93" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D93" s="2">
         <v>1</v>
       </c>
       <c r="E93" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F93" s="2" t="str">
@@ -1808,14 +1798,14 @@
         <v>1</v>
       </c>
       <c r="C94" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D94" s="2">
         <v>1</v>
       </c>
       <c r="E94" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F94" s="2" t="str">
@@ -1831,14 +1821,14 @@
         <v>1</v>
       </c>
       <c r="C95" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D95" s="2">
         <v>1</v>
       </c>
       <c r="E95" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F95" s="2" t="str">
@@ -1854,14 +1844,14 @@
         <v>2</v>
       </c>
       <c r="C96" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D96" s="2">
         <v>2</v>
       </c>
       <c r="E96" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F96" s="2" t="str">
@@ -1877,14 +1867,14 @@
         <v>2</v>
       </c>
       <c r="C97" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D97" s="2">
         <v>2</v>
       </c>
       <c r="E97" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F97" s="2" t="str">
@@ -1900,14 +1890,14 @@
         <v>1</v>
       </c>
       <c r="C98" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D98" s="2">
         <v>1</v>
       </c>
       <c r="E98" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F98" s="2" t="str">
@@ -1923,14 +1913,14 @@
         <v>2</v>
       </c>
       <c r="C99" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D99" s="2">
         <v>2</v>
       </c>
       <c r="E99" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F99" s="2" t="str">
@@ -1946,14 +1936,14 @@
         <v>2</v>
       </c>
       <c r="C100" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D100" s="2">
         <v>2</v>
       </c>
       <c r="E100" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F100" s="2" t="str">
@@ -1969,14 +1959,14 @@
         <v>2</v>
       </c>
       <c r="C101" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D101" s="2">
         <v>2</v>
       </c>
       <c r="E101" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F101" s="2" t="str">
@@ -1992,14 +1982,14 @@
         <v>2</v>
       </c>
       <c r="C102" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D102" s="2">
         <v>2</v>
       </c>
       <c r="E102" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F102" s="2" t="str">
@@ -2015,14 +2005,14 @@
         <v>1</v>
       </c>
       <c r="C103" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D103" s="2">
         <v>1</v>
       </c>
       <c r="E103" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F103" s="2" t="str">
@@ -2038,14 +2028,14 @@
         <v>1</v>
       </c>
       <c r="C104" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>Sáng</v>
       </c>
       <c r="D104" s="2">
         <v>1</v>
       </c>
       <c r="E104" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F104" s="2" t="str">
@@ -2176,37 +2166,37 @@
   <dimension ref="A4:V73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="10" max="10" customWidth="true" width="24.90625"/>
-    <col min="11" max="11" customWidth="true" width="17.90625"/>
-    <col min="15" max="15" customWidth="true" width="17.453125"/>
-    <col min="17" max="17" customWidth="true" width="19.6328125"/>
-    <col min="18" max="18" customWidth="true" width="24.36328125"/>
-    <col min="19" max="19" customWidth="true" width="23.0"/>
+    <col min="10" max="10" width="24.90625" customWidth="1"/>
+    <col min="11" max="11" width="17.90625" customWidth="1"/>
+    <col min="15" max="15" width="17.453125" customWidth="1"/>
+    <col min="17" max="17" width="19.6328125" customWidth="1"/>
+    <col min="18" max="18" width="24.36328125" customWidth="1"/>
+    <col min="19" max="19" width="23" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="24"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="20"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -2272,17 +2262,17 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>89</v>
@@ -2291,7 +2281,7 @@
         <v>72</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>72</v>
@@ -2300,13 +2290,13 @@
         <v>91</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>72</v>
@@ -2340,7 +2330,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="18"/>
+      <c r="A7" s="21"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -2348,7 +2338,7 @@
         <v>88</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>89</v>
@@ -2360,22 +2350,22 @@
         <v>72</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>91</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>72</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>72</v>
@@ -2406,7 +2396,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="18"/>
+      <c r="A8" s="21"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -2414,7 +2404,7 @@
         <v>72</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>72</v>
@@ -2423,7 +2413,7 @@
         <v>89</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>72</v>
@@ -2432,19 +2422,19 @@
         <v>72</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>72</v>
@@ -2453,7 +2443,7 @@
         <v>72</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="R8" s="1" t="s">
         <v>72</v>
@@ -2472,7 +2462,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="18"/>
+      <c r="A9" s="21"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -2480,7 +2470,7 @@
         <v>72</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>72</v>
@@ -2492,7 +2482,7 @@
         <v>72</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>72</v>
@@ -2504,16 +2494,16 @@
         <v>73</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="N9" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>72</v>
@@ -2522,13 +2512,13 @@
         <v>72</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="S9" s="1" t="s">
         <v>72</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="U9" s="1" t="s">
         <v>72</v>
@@ -2538,7 +2528,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="18"/>
+      <c r="A10" s="21"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -2570,13 +2560,13 @@
         <v>72</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="M10" s="1" t="s">
         <v>72</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>73</v>
@@ -2585,26 +2575,26 @@
         <v>72</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="R10" s="1" t="s">
         <v>72</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -2644,10 +2634,10 @@
         <v>72</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="P11" s="1" t="s">
         <v>72</v>
@@ -2672,7 +2662,7 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="20"/>
+      <c r="A12" s="23"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -2738,7 +2728,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="21"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -2804,28 +2794,28 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="23"/>
-      <c r="V16" s="24"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="19"/>
+      <c r="S16" s="19"/>
+      <c r="T16" s="19"/>
+      <c r="U16" s="19"/>
+      <c r="V16" s="20"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -2891,17 +2881,17 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>89</v>
@@ -2910,7 +2900,7 @@
         <v>72</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>72</v>
@@ -2919,13 +2909,13 @@
         <v>91</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>72</v>
@@ -2959,7 +2949,7 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="18"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -2967,7 +2957,7 @@
         <v>88</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>89</v>
@@ -2979,22 +2969,22 @@
         <v>72</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>91</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="L19" s="1" t="s">
         <v>72</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>72</v>
@@ -3025,7 +3015,7 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="18"/>
+      <c r="A20" s="21"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -3033,7 +3023,7 @@
         <v>72</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>72</v>
@@ -3042,7 +3032,7 @@
         <v>89</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>72</v>
@@ -3051,19 +3041,19 @@
         <v>72</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>72</v>
@@ -3072,7 +3062,7 @@
         <v>72</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="R20" s="1" t="s">
         <v>72</v>
@@ -3091,7 +3081,7 @@
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="18"/>
+      <c r="A21" s="21"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -3099,7 +3089,7 @@
         <v>72</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>72</v>
@@ -3111,7 +3101,7 @@
         <v>72</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>72</v>
@@ -3123,16 +3113,16 @@
         <v>73</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="N21" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>72</v>
@@ -3141,13 +3131,13 @@
         <v>72</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="S21" s="1" t="s">
         <v>72</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="U21" s="1" t="s">
         <v>72</v>
@@ -3157,7 +3147,7 @@
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="18"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -3189,13 +3179,13 @@
         <v>72</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="M22" s="1" t="s">
         <v>72</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>73</v>
@@ -3204,26 +3194,26 @@
         <v>72</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="R22" s="1" t="s">
         <v>72</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="T22" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U22" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="V22" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -3263,7 +3253,7 @@
         <v>72</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="O23" s="1" t="s">
         <v>72</v>
@@ -3291,7 +3281,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="20"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -3357,7 +3347,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="21"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -3423,28 +3413,28 @@
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="23"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="23"/>
-      <c r="T28" s="23"/>
-      <c r="U28" s="23"/>
-      <c r="V28" s="24"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="19"/>
+      <c r="S28" s="19"/>
+      <c r="T28" s="19"/>
+      <c r="U28" s="19"/>
+      <c r="V28" s="20"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -3510,20 +3500,20 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
         <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>72</v>
@@ -3538,23 +3528,23 @@
         <v>72</v>
       </c>
       <c r="J30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N30" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O30" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K30" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L30" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="M30" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N30" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="P30" s="1" t="s">
         <v>72</v>
       </c>
@@ -3568,31 +3558,31 @@
         <v>72</v>
       </c>
       <c r="T30" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="U30" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="V30" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="18"/>
+      <c r="A31" s="21"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>89</v>
@@ -3604,47 +3594,47 @@
         <v>72</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="U31" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L31" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="P31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="R31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="S31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="U31" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="V31" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="18"/>
+      <c r="A32" s="21"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -3652,10 +3642,10 @@
         <v>72</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>72</v>
@@ -3667,7 +3657,7 @@
         <v>89</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>72</v>
@@ -3679,7 +3669,7 @@
         <v>72</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="N32" s="1" t="s">
         <v>72</v>
@@ -3691,7 +3681,7 @@
         <v>72</v>
       </c>
       <c r="Q32" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R32" s="1" t="s">
         <v>72</v>
@@ -3700,17 +3690,17 @@
         <v>72</v>
       </c>
       <c r="T32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U32" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="V32" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="U32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="V32" s="1" t="s">
-        <v>91</v>
-      </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="18"/>
+      <c r="A33" s="21"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -3718,13 +3708,13 @@
         <v>72</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>72</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="G33" s="1" t="s">
         <v>72</v>
@@ -3742,13 +3732,13 @@
         <v>72</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>72</v>
@@ -3757,10 +3747,10 @@
         <v>72</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="S33" s="1" t="s">
         <v>72</v>
@@ -3772,11 +3762,11 @@
         <v>72</v>
       </c>
       <c r="V33" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="18"/>
+      <c r="A34" s="21"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -3790,7 +3780,7 @@
         <v>72</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>72</v>
@@ -3799,22 +3789,22 @@
         <v>72</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>72</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>72</v>
@@ -3826,10 +3816,10 @@
         <v>72</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="T34" s="1" t="s">
         <v>72</v>
@@ -3842,7 +3832,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -3910,7 +3900,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="20"/>
+      <c r="A36" s="23"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -3976,7 +3966,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="21"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -4042,28 +4032,28 @@
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="22" t="s">
+      <c r="C40" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="23"/>
-      <c r="K40" s="23"/>
-      <c r="L40" s="23"/>
-      <c r="M40" s="23"/>
-      <c r="N40" s="23"/>
-      <c r="O40" s="23"/>
-      <c r="P40" s="23"/>
-      <c r="Q40" s="23"/>
-      <c r="R40" s="23"/>
-      <c r="S40" s="23"/>
-      <c r="T40" s="23"/>
-      <c r="U40" s="23"/>
-      <c r="V40" s="24"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
+      <c r="K40" s="19"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="19"/>
+      <c r="N40" s="19"/>
+      <c r="O40" s="19"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="19"/>
+      <c r="R40" s="19"/>
+      <c r="S40" s="19"/>
+      <c r="T40" s="19"/>
+      <c r="U40" s="19"/>
+      <c r="V40" s="20"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -4129,7 +4119,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -4197,7 +4187,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="18"/>
+      <c r="A43" s="21"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -4263,7 +4253,7 @@
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="18"/>
+      <c r="A44" s="21"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -4329,7 +4319,7 @@
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="18"/>
+      <c r="A45" s="21"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -4395,7 +4385,7 @@
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="18"/>
+      <c r="A46" s="21"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -4461,7 +4451,7 @@
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -4529,7 +4519,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="20"/>
+      <c r="A48" s="23"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -4595,7 +4585,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="21"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -4661,28 +4651,28 @@
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="22" t="s">
+      <c r="C52" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="23"/>
-      <c r="E52" s="23"/>
-      <c r="F52" s="23"/>
-      <c r="G52" s="23"/>
-      <c r="H52" s="23"/>
-      <c r="I52" s="23"/>
-      <c r="J52" s="23"/>
-      <c r="K52" s="23"/>
-      <c r="L52" s="23"/>
-      <c r="M52" s="23"/>
-      <c r="N52" s="23"/>
-      <c r="O52" s="23"/>
-      <c r="P52" s="23"/>
-      <c r="Q52" s="23"/>
-      <c r="R52" s="23"/>
-      <c r="S52" s="23"/>
-      <c r="T52" s="23"/>
-      <c r="U52" s="23"/>
-      <c r="V52" s="24"/>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="19"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+      <c r="I52" s="19"/>
+      <c r="J52" s="19"/>
+      <c r="K52" s="19"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
+      <c r="N52" s="19"/>
+      <c r="O52" s="19"/>
+      <c r="P52" s="19"/>
+      <c r="Q52" s="19"/>
+      <c r="R52" s="19"/>
+      <c r="S52" s="19"/>
+      <c r="T52" s="19"/>
+      <c r="U52" s="19"/>
+      <c r="V52" s="20"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -4748,20 +4738,20 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="18" t="s">
+      <c r="A54" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
         <v>1</v>
       </c>
       <c r="C54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E54" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>72</v>
@@ -4776,7 +4766,7 @@
         <v>72</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="K54" s="1" t="s">
         <v>72</v>
@@ -4791,13 +4781,13 @@
         <v>72</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="P54" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q54" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R54" s="1" t="s">
         <v>72</v>
@@ -4809,14 +4799,14 @@
         <v>72</v>
       </c>
       <c r="U54" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="V54" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="18"/>
+      <c r="A55" s="21"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -4824,13 +4814,13 @@
         <v>72</v>
       </c>
       <c r="D55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>72</v>
@@ -4845,7 +4835,7 @@
         <v>72</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="L55" s="1" t="s">
         <v>72</v>
@@ -4863,7 +4853,7 @@
         <v>72</v>
       </c>
       <c r="Q55" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R55" s="1" t="s">
         <v>72</v>
@@ -4872,17 +4862,17 @@
         <v>72</v>
       </c>
       <c r="T55" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="U55" s="1" t="s">
         <v>72</v>
       </c>
       <c r="V55" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="18"/>
+      <c r="A56" s="21"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -4893,19 +4883,19 @@
         <v>72</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I56" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I56" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="J56" s="1" t="s">
         <v>72</v>
@@ -4923,7 +4913,7 @@
         <v>88</v>
       </c>
       <c r="O56" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P56" s="1" t="s">
         <v>72</v>
@@ -4932,23 +4922,23 @@
         <v>72</v>
       </c>
       <c r="R56" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S56" s="1" t="s">
         <v>72</v>
       </c>
       <c r="T56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="V56" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="U56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="V56" s="1" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="18"/>
+      <c r="A57" s="21"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -4962,10 +4952,10 @@
         <v>72</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="H57" s="1" t="s">
         <v>72</v>
@@ -4995,10 +4985,10 @@
         <v>72</v>
       </c>
       <c r="Q57" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R57" s="1" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="S57" s="1" t="s">
         <v>72</v>
@@ -5007,14 +4997,14 @@
         <v>72</v>
       </c>
       <c r="U57" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="V57" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="18"/>
+      <c r="A58" s="21"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -5037,38 +5027,38 @@
         <v>72</v>
       </c>
       <c r="I58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L58" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="M58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q58" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S58" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="J58" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K58" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L58" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="M58" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N58" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O58" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="P58" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q58" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="R58" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="S58" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="T58" s="1" t="s">
         <v>72</v>
       </c>
@@ -5076,11 +5066,11 @@
         <v>72</v>
       </c>
       <c r="V58" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -5148,7 +5138,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="20"/>
+      <c r="A60" s="23"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -5214,7 +5204,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="21"/>
+      <c r="A61" s="24"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -5280,28 +5270,28 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="22" t="s">
+      <c r="C64" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="23"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="23"/>
-      <c r="G64" s="23"/>
-      <c r="H64" s="23"/>
-      <c r="I64" s="23"/>
-      <c r="J64" s="23"/>
-      <c r="K64" s="23"/>
-      <c r="L64" s="23"/>
-      <c r="M64" s="23"/>
-      <c r="N64" s="23"/>
-      <c r="O64" s="23"/>
-      <c r="P64" s="23"/>
-      <c r="Q64" s="23"/>
-      <c r="R64" s="23"/>
-      <c r="S64" s="23"/>
-      <c r="T64" s="23"/>
-      <c r="U64" s="23"/>
-      <c r="V64" s="24"/>
+      <c r="D64" s="19"/>
+      <c r="E64" s="19"/>
+      <c r="F64" s="19"/>
+      <c r="G64" s="19"/>
+      <c r="H64" s="19"/>
+      <c r="I64" s="19"/>
+      <c r="J64" s="19"/>
+      <c r="K64" s="19"/>
+      <c r="L64" s="19"/>
+      <c r="M64" s="19"/>
+      <c r="N64" s="19"/>
+      <c r="O64" s="19"/>
+      <c r="P64" s="19"/>
+      <c r="Q64" s="19"/>
+      <c r="R64" s="19"/>
+      <c r="S64" s="19"/>
+      <c r="T64" s="19"/>
+      <c r="U64" s="19"/>
+      <c r="V64" s="20"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -5367,7 +5357,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="18" t="s">
+      <c r="A66" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -5389,10 +5379,10 @@
         <v>72</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="J66" s="1" t="s">
         <v>72</v>
@@ -5404,10 +5394,10 @@
         <v>72</v>
       </c>
       <c r="M66" s="1" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="O66" s="1" t="s">
         <v>72</v>
@@ -5416,26 +5406,26 @@
         <v>72</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R66" s="1" t="s">
         <v>72</v>
       </c>
       <c r="S66" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="T66" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="U66" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="V66" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="18"/>
+      <c r="A67" s="21"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -5449,13 +5439,13 @@
         <v>72</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="G67" s="1" t="s">
         <v>72</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>72</v>
@@ -5467,13 +5457,13 @@
         <v>72</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="O67" s="1" t="s">
         <v>72</v>
@@ -5482,26 +5472,26 @@
         <v>72</v>
       </c>
       <c r="Q67" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R67" s="1" t="s">
         <v>72</v>
       </c>
       <c r="S67" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="T67" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U67" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="V67" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="18"/>
+      <c r="A68" s="21"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -5515,7 +5505,7 @@
         <v>72</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>72</v>
@@ -5533,17 +5523,17 @@
         <v>72</v>
       </c>
       <c r="L68" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M68" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="N68" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O68" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="M68" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N68" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="O68" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="P68" s="1" t="s">
         <v>72</v>
       </c>
@@ -5551,7 +5541,7 @@
         <v>72</v>
       </c>
       <c r="R68" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S68" s="1" t="s">
         <v>72</v>
@@ -5563,11 +5553,11 @@
         <v>72</v>
       </c>
       <c r="V68" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="18"/>
+      <c r="A69" s="21"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -5584,7 +5574,7 @@
         <v>72</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="H69" s="1" t="s">
         <v>72</v>
@@ -5602,13 +5592,13 @@
         <v>72</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="P69" s="1" t="s">
         <v>72</v>
@@ -5629,11 +5619,11 @@
         <v>72</v>
       </c>
       <c r="V69" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="18"/>
+      <c r="A70" s="21"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -5650,13 +5640,13 @@
         <v>72</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="H70" s="1" t="s">
         <v>72</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="J70" s="1" t="s">
         <v>72</v>
@@ -5699,7 +5689,7 @@
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="19" t="s">
+      <c r="A71" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -5767,7 +5757,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="20"/>
+      <c r="A72" s="23"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -5833,7 +5823,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="21"/>
+      <c r="A73" s="24"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -5900,16 +5890,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -5918,6 +5898,16 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixed adding enough lesson per week
</commit_message>
<xml_diff>
--- a/bin/excel_resources/excel_data.xlsx
+++ b/bin/excel_resources/excel_data.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA6B1EB5-25AE-4BB2-9D19-D0E02F79F37E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95676F4-FDF9-4DED-9845-F83B0BC78DE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2167" uniqueCount="107">
   <si>
     <t>10A1</t>
   </si>
@@ -337,9 +337,6 @@
     <t>Tiết học tránh dạy (T7)</t>
   </si>
   <si>
-    <t>3,4</t>
-  </si>
-  <si>
     <t>2,3</t>
   </si>
   <si>
@@ -347,12 +344,16 @@
   </si>
   <si>
     <t>Mã Đức Bảo-CD Văn</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Hằng-CD Sử</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -548,15 +549,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -568,6 +560,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -852,25 +853,25 @@
   <dimension ref="A5:U124"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.08984375" customWidth="1"/>
-    <col min="2" max="2" width="63.08984375" customWidth="1"/>
-    <col min="3" max="3" width="20.1796875" customWidth="1"/>
-    <col min="4" max="4" width="16.36328125" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" customWidth="1"/>
-    <col min="6" max="6" width="22.7265625" customWidth="1"/>
-    <col min="7" max="7" width="21.54296875" customWidth="1"/>
-    <col min="8" max="8" width="20.36328125" customWidth="1"/>
-    <col min="9" max="9" width="26.453125" customWidth="1"/>
-    <col min="10" max="10" width="22.81640625" customWidth="1"/>
-    <col min="11" max="11" width="23.36328125" customWidth="1"/>
-    <col min="12" max="12" width="12.7265625" customWidth="1"/>
-    <col min="13" max="13" width="19.1796875" customWidth="1"/>
-    <col min="14" max="14" width="16.08984375" customWidth="1"/>
-    <col min="15" max="15" width="16.1796875" customWidth="1"/>
-    <col min="16" max="16" width="10.90625" customWidth="1"/>
-    <col min="17" max="17" width="13.54296875" customWidth="1"/>
-    <col min="20" max="20" width="17.08984375" customWidth="1"/>
-    <col min="21" max="21" width="9.90625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="28.08984375"/>
+    <col min="2" max="2" customWidth="true" width="63.08984375"/>
+    <col min="3" max="3" customWidth="true" width="20.1796875"/>
+    <col min="4" max="4" customWidth="true" width="16.36328125"/>
+    <col min="5" max="5" customWidth="true" width="15.26953125"/>
+    <col min="6" max="6" customWidth="true" width="22.7265625"/>
+    <col min="7" max="7" customWidth="true" width="21.54296875"/>
+    <col min="8" max="8" customWidth="true" width="20.36328125"/>
+    <col min="9" max="9" customWidth="true" width="26.453125"/>
+    <col min="10" max="10" customWidth="true" width="22.81640625"/>
+    <col min="11" max="11" customWidth="true" width="23.36328125"/>
+    <col min="12" max="12" customWidth="true" width="12.7265625"/>
+    <col min="13" max="13" customWidth="true" width="19.1796875"/>
+    <col min="14" max="14" customWidth="true" width="16.08984375"/>
+    <col min="15" max="15" customWidth="true" width="16.1796875"/>
+    <col min="16" max="16" customWidth="true" width="10.90625"/>
+    <col min="17" max="17" customWidth="true" width="13.54296875"/>
+    <col min="20" max="20" customWidth="true" width="17.08984375"/>
+    <col min="21" max="21" customWidth="true" width="9.90625"/>
   </cols>
   <sheetData>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -968,22 +969,12 @@
       <c r="E8" s="13">
         <v>35</v>
       </c>
-      <c r="F8" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>103</v>
-      </c>
+      <c r="F8" s="13"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>96</v>
-      </c>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
       <c r="L8" s="13" t="str">
         <f t="shared" ref="L8:L18" si="1">A$117</f>
         <v>Thứ Năm</v>
@@ -1021,7 +1012,7 @@
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>95</v>
@@ -2166,37 +2157,37 @@
   <dimension ref="A4:V73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="10" max="10" width="24.90625" customWidth="1"/>
-    <col min="11" max="11" width="17.90625" customWidth="1"/>
-    <col min="15" max="15" width="17.453125" customWidth="1"/>
-    <col min="17" max="17" width="19.6328125" customWidth="1"/>
-    <col min="18" max="18" width="24.36328125" customWidth="1"/>
-    <col min="19" max="19" width="23" customWidth="1"/>
+    <col min="10" max="10" customWidth="true" width="24.90625"/>
+    <col min="11" max="11" customWidth="true" width="17.90625"/>
+    <col min="15" max="15" customWidth="true" width="17.453125"/>
+    <col min="17" max="17" customWidth="true" width="19.6328125"/>
+    <col min="18" max="18" customWidth="true" width="24.36328125"/>
+    <col min="19" max="19" customWidth="true" width="23.0"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="20"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="23"/>
+      <c r="T4" s="23"/>
+      <c r="U4" s="23"/>
+      <c r="V4" s="24"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -2262,7 +2253,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -2293,7 +2284,7 @@
         <v>92</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>72</v>
@@ -2330,7 +2321,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="21"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -2356,7 +2347,7 @@
         <v>91</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>92</v>
@@ -2396,7 +2387,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="21"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -2422,7 +2413,7 @@
         <v>72</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>72</v>
@@ -2437,7 +2428,7 @@
         <v>72</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>72</v>
@@ -2462,7 +2453,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="21"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -2491,7 +2482,7 @@
         <v>72</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>88</v>
@@ -2503,7 +2494,7 @@
         <v>72</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>72</v>
@@ -2528,7 +2519,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="21"/>
+      <c r="A10" s="18"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -2569,17 +2560,17 @@
         <v>92</v>
       </c>
       <c r="O10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q10" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="P10" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q10" s="1" t="s">
+      <c r="R10" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="R10" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="S10" s="1" t="s">
         <v>72</v>
       </c>
@@ -2594,7 +2585,7 @@
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -2637,7 +2628,7 @@
         <v>93</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="P11" s="1" t="s">
         <v>72</v>
@@ -2662,7 +2653,7 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="23"/>
+      <c r="A12" s="20"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -2728,7 +2719,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="24"/>
+      <c r="A13" s="21"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -2794,28 +2785,28 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
-      <c r="O16" s="19"/>
-      <c r="P16" s="19"/>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="19"/>
-      <c r="S16" s="19"/>
-      <c r="T16" s="19"/>
-      <c r="U16" s="19"/>
-      <c r="V16" s="20"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+      <c r="R16" s="23"/>
+      <c r="S16" s="23"/>
+      <c r="T16" s="23"/>
+      <c r="U16" s="23"/>
+      <c r="V16" s="24"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -2881,7 +2872,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
@@ -2912,7 +2903,7 @@
         <v>92</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L18" s="1" t="s">
         <v>72</v>
@@ -2949,7 +2940,7 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="21"/>
+      <c r="A19" s="18"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -2975,7 +2966,7 @@
         <v>91</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>92</v>
@@ -3015,7 +3006,7 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="21"/>
+      <c r="A20" s="18"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -3041,7 +3032,7 @@
         <v>72</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>72</v>
@@ -3056,7 +3047,7 @@
         <v>72</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>72</v>
@@ -3081,7 +3072,7 @@
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="21"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -3110,7 +3101,7 @@
         <v>72</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L21" s="1" t="s">
         <v>88</v>
@@ -3122,7 +3113,7 @@
         <v>72</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>72</v>
@@ -3147,7 +3138,7 @@
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="21"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -3188,17 +3179,17 @@
         <v>92</v>
       </c>
       <c r="O22" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q22" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="P22" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q22" s="1" t="s">
+      <c r="R22" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="R22" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="S22" s="1" t="s">
         <v>72</v>
       </c>
@@ -3213,7 +3204,7 @@
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -3253,7 +3244,7 @@
         <v>72</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O23" s="1" t="s">
         <v>72</v>
@@ -3281,7 +3272,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="23"/>
+      <c r="A24" s="20"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -3347,7 +3338,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="24"/>
+      <c r="A25" s="21"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -3413,28 +3404,28 @@
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="19"/>
-      <c r="O28" s="19"/>
-      <c r="P28" s="19"/>
-      <c r="Q28" s="19"/>
-      <c r="R28" s="19"/>
-      <c r="S28" s="19"/>
-      <c r="T28" s="19"/>
-      <c r="U28" s="19"/>
-      <c r="V28" s="20"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="23"/>
+      <c r="N28" s="23"/>
+      <c r="O28" s="23"/>
+      <c r="P28" s="23"/>
+      <c r="Q28" s="23"/>
+      <c r="R28" s="23"/>
+      <c r="S28" s="23"/>
+      <c r="T28" s="23"/>
+      <c r="U28" s="23"/>
+      <c r="V28" s="24"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -3500,7 +3491,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="21" t="s">
+      <c r="A30" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -3568,7 +3559,7 @@
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="21"/>
+      <c r="A31" s="18"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -3634,7 +3625,7 @@
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="21"/>
+      <c r="A32" s="18"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -3663,7 +3654,7 @@
         <v>72</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L32" s="1" t="s">
         <v>72</v>
@@ -3700,7 +3691,7 @@
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="21"/>
+      <c r="A33" s="18"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -3729,7 +3720,7 @@
         <v>72</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L33" s="1" t="s">
         <v>93</v>
@@ -3747,10 +3738,10 @@
         <v>72</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="S33" s="1" t="s">
         <v>72</v>
@@ -3766,7 +3757,7 @@
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="21"/>
+      <c r="A34" s="18"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -3795,7 +3786,7 @@
         <v>72</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L34" s="1" t="s">
         <v>88</v>
@@ -3813,7 +3804,7 @@
         <v>72</v>
       </c>
       <c r="Q34" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R34" s="1" t="s">
         <v>72</v>
@@ -3832,7 +3823,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -3857,7 +3848,7 @@
         <v>72</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>72</v>
@@ -3900,7 +3891,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="23"/>
+      <c r="A36" s="20"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -3966,7 +3957,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="24"/>
+      <c r="A37" s="21"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -4032,28 +4023,28 @@
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="18" t="s">
+      <c r="C40" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="19"/>
-      <c r="J40" s="19"/>
-      <c r="K40" s="19"/>
-      <c r="L40" s="19"/>
-      <c r="M40" s="19"/>
-      <c r="N40" s="19"/>
-      <c r="O40" s="19"/>
-      <c r="P40" s="19"/>
-      <c r="Q40" s="19"/>
-      <c r="R40" s="19"/>
-      <c r="S40" s="19"/>
-      <c r="T40" s="19"/>
-      <c r="U40" s="19"/>
-      <c r="V40" s="20"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
+      <c r="J40" s="23"/>
+      <c r="K40" s="23"/>
+      <c r="L40" s="23"/>
+      <c r="M40" s="23"/>
+      <c r="N40" s="23"/>
+      <c r="O40" s="23"/>
+      <c r="P40" s="23"/>
+      <c r="Q40" s="23"/>
+      <c r="R40" s="23"/>
+      <c r="S40" s="23"/>
+      <c r="T40" s="23"/>
+      <c r="U40" s="23"/>
+      <c r="V40" s="24"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -4119,7 +4110,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="21" t="s">
+      <c r="A42" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -4187,7 +4178,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="21"/>
+      <c r="A43" s="18"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -4253,7 +4244,7 @@
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="21"/>
+      <c r="A44" s="18"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -4319,7 +4310,7 @@
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="21"/>
+      <c r="A45" s="18"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -4385,7 +4376,7 @@
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="21"/>
+      <c r="A46" s="18"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -4451,7 +4442,7 @@
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="22" t="s">
+      <c r="A47" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -4519,7 +4510,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="23"/>
+      <c r="A48" s="20"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -4585,7 +4576,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="24"/>
+      <c r="A49" s="21"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -4651,28 +4642,28 @@
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="18" t="s">
+      <c r="C52" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="19"/>
-      <c r="E52" s="19"/>
-      <c r="F52" s="19"/>
-      <c r="G52" s="19"/>
-      <c r="H52" s="19"/>
-      <c r="I52" s="19"/>
-      <c r="J52" s="19"/>
-      <c r="K52" s="19"/>
-      <c r="L52" s="19"/>
-      <c r="M52" s="19"/>
-      <c r="N52" s="19"/>
-      <c r="O52" s="19"/>
-      <c r="P52" s="19"/>
-      <c r="Q52" s="19"/>
-      <c r="R52" s="19"/>
-      <c r="S52" s="19"/>
-      <c r="T52" s="19"/>
-      <c r="U52" s="19"/>
-      <c r="V52" s="20"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="23"/>
+      <c r="I52" s="23"/>
+      <c r="J52" s="23"/>
+      <c r="K52" s="23"/>
+      <c r="L52" s="23"/>
+      <c r="M52" s="23"/>
+      <c r="N52" s="23"/>
+      <c r="O52" s="23"/>
+      <c r="P52" s="23"/>
+      <c r="Q52" s="23"/>
+      <c r="R52" s="23"/>
+      <c r="S52" s="23"/>
+      <c r="T52" s="23"/>
+      <c r="U52" s="23"/>
+      <c r="V52" s="24"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -4738,7 +4729,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="21" t="s">
+      <c r="A54" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
@@ -4790,7 +4781,7 @@
         <v>72</v>
       </c>
       <c r="R54" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S54" s="1" t="s">
         <v>72</v>
@@ -4806,7 +4797,7 @@
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="21"/>
+      <c r="A55" s="18"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -4856,7 +4847,7 @@
         <v>72</v>
       </c>
       <c r="R55" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S55" s="1" t="s">
         <v>72</v>
@@ -4872,7 +4863,7 @@
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="21"/>
+      <c r="A56" s="18"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -4913,19 +4904,19 @@
         <v>88</v>
       </c>
       <c r="O56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S56" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="P56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="R56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="S56" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="T56" s="1" t="s">
         <v>72</v>
@@ -4938,7 +4929,7 @@
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="21"/>
+      <c r="A57" s="18"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -4979,19 +4970,19 @@
         <v>88</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="P57" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q57" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="R57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S57" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="R57" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="S57" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="T57" s="1" t="s">
         <v>72</v>
@@ -5004,7 +4995,7 @@
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="21"/>
+      <c r="A58" s="18"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -5018,7 +5009,7 @@
         <v>72</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>72</v>
@@ -5036,7 +5027,7 @@
         <v>72</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M58" s="1" t="s">
         <v>72</v>
@@ -5051,13 +5042,13 @@
         <v>72</v>
       </c>
       <c r="Q58" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R58" s="1" t="s">
         <v>72</v>
       </c>
       <c r="S58" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="T58" s="1" t="s">
         <v>72</v>
@@ -5070,7 +5061,7 @@
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="22" t="s">
+      <c r="A59" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -5138,7 +5129,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="23"/>
+      <c r="A60" s="20"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -5204,7 +5195,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="24"/>
+      <c r="A61" s="21"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -5270,28 +5261,28 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="18" t="s">
+      <c r="C64" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="19"/>
-      <c r="E64" s="19"/>
-      <c r="F64" s="19"/>
-      <c r="G64" s="19"/>
-      <c r="H64" s="19"/>
-      <c r="I64" s="19"/>
-      <c r="J64" s="19"/>
-      <c r="K64" s="19"/>
-      <c r="L64" s="19"/>
-      <c r="M64" s="19"/>
-      <c r="N64" s="19"/>
-      <c r="O64" s="19"/>
-      <c r="P64" s="19"/>
-      <c r="Q64" s="19"/>
-      <c r="R64" s="19"/>
-      <c r="S64" s="19"/>
-      <c r="T64" s="19"/>
-      <c r="U64" s="19"/>
-      <c r="V64" s="20"/>
+      <c r="D64" s="23"/>
+      <c r="E64" s="23"/>
+      <c r="F64" s="23"/>
+      <c r="G64" s="23"/>
+      <c r="H64" s="23"/>
+      <c r="I64" s="23"/>
+      <c r="J64" s="23"/>
+      <c r="K64" s="23"/>
+      <c r="L64" s="23"/>
+      <c r="M64" s="23"/>
+      <c r="N64" s="23"/>
+      <c r="O64" s="23"/>
+      <c r="P64" s="23"/>
+      <c r="Q64" s="23"/>
+      <c r="R64" s="23"/>
+      <c r="S64" s="23"/>
+      <c r="T64" s="23"/>
+      <c r="U64" s="23"/>
+      <c r="V64" s="24"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -5357,7 +5348,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="21" t="s">
+      <c r="A66" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -5376,7 +5367,7 @@
         <v>72</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="H66" s="1" t="s">
         <v>72</v>
@@ -5406,10 +5397,10 @@
         <v>72</v>
       </c>
       <c r="Q66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R66" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="R66" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="S66" s="1" t="s">
         <v>72</v>
@@ -5425,7 +5416,7 @@
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="21"/>
+      <c r="A67" s="18"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -5442,7 +5433,7 @@
         <v>72</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="H67" s="1" t="s">
         <v>72</v>
@@ -5472,10 +5463,10 @@
         <v>72</v>
       </c>
       <c r="Q67" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R67" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="R67" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="S67" s="1" t="s">
         <v>72</v>
@@ -5491,7 +5482,7 @@
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="21"/>
+      <c r="A68" s="18"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -5511,7 +5502,7 @@
         <v>72</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>72</v>
@@ -5526,13 +5517,13 @@
         <v>72</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N68" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="P68" s="1" t="s">
         <v>72</v>
@@ -5541,10 +5532,10 @@
         <v>72</v>
       </c>
       <c r="R68" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S68" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="S68" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="T68" s="1" t="s">
         <v>72</v>
@@ -5557,7 +5548,7 @@
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="21"/>
+      <c r="A69" s="18"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -5577,7 +5568,7 @@
         <v>72</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>72</v>
@@ -5592,13 +5583,13 @@
         <v>72</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N69" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="P69" s="1" t="s">
         <v>72</v>
@@ -5610,7 +5601,7 @@
         <v>72</v>
       </c>
       <c r="S69" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="T69" s="1" t="s">
         <v>72</v>
@@ -5623,7 +5614,7 @@
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="21"/>
+      <c r="A70" s="18"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -5664,7 +5655,7 @@
         <v>72</v>
       </c>
       <c r="O70" s="1" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="P70" s="1" t="s">
         <v>72</v>
@@ -5689,7 +5680,7 @@
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="22" t="s">
+      <c r="A71" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -5757,7 +5748,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="23"/>
+      <c r="A72" s="20"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -5823,7 +5814,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="24"/>
+      <c r="A73" s="21"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -5890,6 +5881,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -5898,16 +5899,6 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
revise distribution lessons equally
</commit_message>
<xml_diff>
--- a/bin/excel_resources/excel_data.xlsx
+++ b/bin/excel_resources/excel_data.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95676F4-FDF9-4DED-9845-F83B0BC78DE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC59CBD-F45D-4193-AA5A-7290932A14D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2167" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="105">
   <si>
     <t>10A1</t>
   </si>
@@ -310,9 +310,6 @@
     <t>Hoàng Văn Chinh-CD Sử</t>
   </si>
   <si>
-    <t>Hoàng Hiếu Trình-CD Văn</t>
-  </si>
-  <si>
     <t>1,2</t>
   </si>
   <si>
@@ -340,20 +337,16 @@
     <t>2,3</t>
   </si>
   <si>
-    <t>Vi Văn Tình-CD Văn</t>
-  </si>
-  <si>
-    <t>Mã Đức Bảo-CD Văn</t>
-  </si>
-  <si>
     <t>Nguyễn Thị Hằng-CD Sử</t>
+  </si>
+  <si>
+    <t>Cao Thị Tố Uyên-CD Văn</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -549,6 +542,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -560,15 +562,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -853,25 +846,25 @@
   <dimension ref="A5:U124"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="28.08984375"/>
-    <col min="2" max="2" customWidth="true" width="63.08984375"/>
-    <col min="3" max="3" customWidth="true" width="20.1796875"/>
-    <col min="4" max="4" customWidth="true" width="16.36328125"/>
-    <col min="5" max="5" customWidth="true" width="15.26953125"/>
-    <col min="6" max="6" customWidth="true" width="22.7265625"/>
-    <col min="7" max="7" customWidth="true" width="21.54296875"/>
-    <col min="8" max="8" customWidth="true" width="20.36328125"/>
-    <col min="9" max="9" customWidth="true" width="26.453125"/>
-    <col min="10" max="10" customWidth="true" width="22.81640625"/>
-    <col min="11" max="11" customWidth="true" width="23.36328125"/>
-    <col min="12" max="12" customWidth="true" width="12.7265625"/>
-    <col min="13" max="13" customWidth="true" width="19.1796875"/>
-    <col min="14" max="14" customWidth="true" width="16.08984375"/>
-    <col min="15" max="15" customWidth="true" width="16.1796875"/>
-    <col min="16" max="16" customWidth="true" width="10.90625"/>
-    <col min="17" max="17" customWidth="true" width="13.54296875"/>
-    <col min="20" max="20" customWidth="true" width="17.08984375"/>
-    <col min="21" max="21" customWidth="true" width="9.90625"/>
+    <col min="1" max="1" width="28.08984375" customWidth="1"/>
+    <col min="2" max="2" width="63.08984375" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" customWidth="1"/>
+    <col min="6" max="6" width="22.7265625" customWidth="1"/>
+    <col min="7" max="7" width="21.54296875" customWidth="1"/>
+    <col min="8" max="8" width="20.36328125" customWidth="1"/>
+    <col min="9" max="9" width="26.453125" customWidth="1"/>
+    <col min="10" max="10" width="22.81640625" customWidth="1"/>
+    <col min="11" max="11" width="23.36328125" customWidth="1"/>
+    <col min="12" max="12" width="12.7265625" customWidth="1"/>
+    <col min="13" max="13" width="19.1796875" customWidth="1"/>
+    <col min="14" max="14" width="16.08984375" customWidth="1"/>
+    <col min="15" max="15" width="16.1796875" customWidth="1"/>
+    <col min="16" max="16" width="10.90625" customWidth="1"/>
+    <col min="17" max="17" width="13.54296875" customWidth="1"/>
+    <col min="20" max="20" width="17.08984375" customWidth="1"/>
+    <col min="21" max="21" width="9.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -896,22 +889,22 @@
         <v>32</v>
       </c>
       <c r="F6" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="G6" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="H6" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="H6" s="16" t="s">
+      <c r="I6" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="I6" s="14" t="s">
+      <c r="J6" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="J6" s="16" t="s">
+      <c r="K6" s="16" t="s">
         <v>101</v>
-      </c>
-      <c r="K6" s="16" t="s">
-        <v>102</v>
       </c>
       <c r="L6" s="14" t="s">
         <v>62</v>
@@ -944,11 +937,11 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="13" t="str">
-        <f>A117</f>
+        <f t="shared" ref="L7:L18" si="0">A$117</f>
         <v>Thứ Năm</v>
       </c>
       <c r="M7" s="13" t="str">
-        <f t="shared" ref="M7:M18" si="0">F$89</f>
+        <f t="shared" ref="M7:M18" si="1">F$89</f>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -976,11 +969,11 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="13" t="str">
-        <f t="shared" ref="L8:L18" si="1">A$117</f>
+        <f t="shared" si="0"/>
         <v>Thứ Năm</v>
       </c>
       <c r="M8" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1002,27 +995,27 @@
         <v>105</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L9" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M9" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M9" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1049,11 +1042,11 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M10" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M10" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1081,11 +1074,11 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M11" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M11" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1112,11 +1105,11 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M12" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M12" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1144,11 +1137,11 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M13" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M13" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1175,11 +1168,11 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M14" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M14" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1207,11 +1200,11 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
       <c r="L15" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M15" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M15" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1239,11 +1232,11 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
       <c r="L16" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M16" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M16" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1271,11 +1264,11 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M17" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M17" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -1303,11 +1296,11 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>Thứ Năm</v>
+      </c>
+      <c r="M18" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>Thứ Năm</v>
-      </c>
-      <c r="M18" s="13" t="str">
-        <f t="shared" si="0"/>
         <v>Xã Hội</v>
       </c>
     </row>
@@ -2157,37 +2150,37 @@
   <dimension ref="A4:V73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="10" max="10" customWidth="true" width="24.90625"/>
-    <col min="11" max="11" customWidth="true" width="17.90625"/>
-    <col min="15" max="15" customWidth="true" width="17.453125"/>
-    <col min="17" max="17" customWidth="true" width="19.6328125"/>
-    <col min="18" max="18" customWidth="true" width="24.36328125"/>
-    <col min="19" max="19" customWidth="true" width="23.0"/>
+    <col min="10" max="10" width="24.90625" customWidth="1"/>
+    <col min="11" max="11" width="17.90625" customWidth="1"/>
+    <col min="15" max="15" width="17.453125" customWidth="1"/>
+    <col min="17" max="17" width="19.6328125" customWidth="1"/>
+    <col min="18" max="18" width="24.36328125" customWidth="1"/>
+    <col min="19" max="19" width="23" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="24"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="20"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -2253,7 +2246,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -2321,7 +2314,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="18"/>
+      <c r="A7" s="21"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -2387,7 +2380,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="18"/>
+      <c r="A8" s="21"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -2401,10 +2394,10 @@
         <v>72</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>72</v>
@@ -2422,7 +2415,7 @@
         <v>92</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>72</v>
@@ -2443,7 +2436,7 @@
         <v>72</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="U8" s="1" t="s">
         <v>72</v>
@@ -2453,7 +2446,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="18"/>
+      <c r="A9" s="21"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -2467,13 +2460,13 @@
         <v>72</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>72</v>
@@ -2488,13 +2481,13 @@
         <v>88</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N9" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>72</v>
@@ -2519,7 +2512,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="18"/>
+      <c r="A10" s="21"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -2536,7 +2529,7 @@
         <v>72</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>72</v>
@@ -2557,7 +2550,7 @@
         <v>72</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>72</v>
@@ -2566,10 +2559,10 @@
         <v>72</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="S10" s="1" t="s">
         <v>72</v>
@@ -2585,7 +2578,7 @@
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -2625,7 +2618,7 @@
         <v>72</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>72</v>
@@ -2653,7 +2646,7 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="20"/>
+      <c r="A12" s="23"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -2719,7 +2712,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="21"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -2785,28 +2778,28 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="23"/>
-      <c r="V16" s="24"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="19"/>
+      <c r="S16" s="19"/>
+      <c r="T16" s="19"/>
+      <c r="U16" s="19"/>
+      <c r="V16" s="20"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -2872,7 +2865,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
@@ -2940,7 +2933,7 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="18"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -2951,11 +2944,11 @@
         <v>90</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="G19" s="1" t="s">
         <v>72</v>
       </c>
@@ -2963,7 +2956,7 @@
         <v>72</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>73</v>
@@ -2996,7 +2989,7 @@
         <v>72</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="U19" s="1" t="s">
         <v>72</v>
@@ -3006,7 +2999,7 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="18"/>
+      <c r="A20" s="21"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -3017,13 +3010,13 @@
         <v>72</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>72</v>
@@ -3041,7 +3034,7 @@
         <v>92</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="N20" s="1" t="s">
         <v>72</v>
@@ -3062,7 +3055,7 @@
         <v>72</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="U20" s="1" t="s">
         <v>72</v>
@@ -3072,7 +3065,7 @@
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="18"/>
+      <c r="A21" s="21"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -3086,13 +3079,13 @@
         <v>72</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>72</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>72</v>
@@ -3113,7 +3106,7 @@
         <v>72</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>72</v>
@@ -3138,7 +3131,7 @@
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="18"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -3155,7 +3148,7 @@
         <v>72</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>72</v>
@@ -3176,7 +3169,7 @@
         <v>72</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>72</v>
@@ -3185,10 +3178,10 @@
         <v>72</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="S22" s="1" t="s">
         <v>72</v>
@@ -3204,7 +3197,7 @@
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -3244,7 +3237,7 @@
         <v>72</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="O23" s="1" t="s">
         <v>72</v>
@@ -3272,7 +3265,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="20"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -3338,7 +3331,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="21"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -3404,28 +3397,28 @@
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="23"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="23"/>
-      <c r="T28" s="23"/>
-      <c r="U28" s="23"/>
-      <c r="V28" s="24"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="19"/>
+      <c r="S28" s="19"/>
+      <c r="T28" s="19"/>
+      <c r="U28" s="19"/>
+      <c r="V28" s="20"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -3491,7 +3484,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -3507,10 +3500,10 @@
         <v>90</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>72</v>
@@ -3528,13 +3521,13 @@
         <v>72</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="N30" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="P30" s="1" t="s">
         <v>72</v>
@@ -3559,25 +3552,25 @@
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="18"/>
+      <c r="A31" s="21"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="E31" s="1" t="s">
         <v>72</v>
       </c>
       <c r="F31" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G31" s="1" t="s">
-        <v>89</v>
-      </c>
       <c r="H31" s="1" t="s">
         <v>72</v>
       </c>
@@ -3585,11 +3578,11 @@
         <v>72</v>
       </c>
       <c r="J31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K31" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="K31" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="L31" s="1" t="s">
         <v>72</v>
       </c>
@@ -3597,7 +3590,7 @@
         <v>72</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>72</v>
@@ -3618,14 +3611,14 @@
         <v>91</v>
       </c>
       <c r="U31" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="V31" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="18"/>
+      <c r="A32" s="21"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -3633,32 +3626,32 @@
         <v>72</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L32" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L32" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="M32" s="1" t="s">
         <v>72</v>
       </c>
@@ -3666,7 +3659,7 @@
         <v>72</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="P32" s="1" t="s">
         <v>72</v>
@@ -3684,14 +3677,14 @@
         <v>72</v>
       </c>
       <c r="U32" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="V32" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="18"/>
+      <c r="A33" s="21"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -3699,7 +3692,7 @@
         <v>72</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>72</v>
@@ -3711,34 +3704,34 @@
         <v>72</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>72</v>
       </c>
       <c r="K33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O33" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="L33" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="M33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="P33" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="R33" s="1" t="s">
         <v>72</v>
@@ -3750,14 +3743,14 @@
         <v>72</v>
       </c>
       <c r="U33" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="V33" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="18"/>
+      <c r="A34" s="21"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -3789,10 +3782,10 @@
         <v>72</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="N34" s="1" t="s">
         <v>72</v>
@@ -3804,13 +3797,13 @@
         <v>72</v>
       </c>
       <c r="Q34" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R34" s="1" t="s">
         <v>72</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="T34" s="1" t="s">
         <v>72</v>
@@ -3823,7 +3816,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -3848,7 +3841,7 @@
         <v>72</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>72</v>
@@ -3891,7 +3884,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="20"/>
+      <c r="A36" s="23"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -3957,7 +3950,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="21"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -4023,28 +4016,28 @@
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="22" t="s">
+      <c r="C40" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="23"/>
-      <c r="K40" s="23"/>
-      <c r="L40" s="23"/>
-      <c r="M40" s="23"/>
-      <c r="N40" s="23"/>
-      <c r="O40" s="23"/>
-      <c r="P40" s="23"/>
-      <c r="Q40" s="23"/>
-      <c r="R40" s="23"/>
-      <c r="S40" s="23"/>
-      <c r="T40" s="23"/>
-      <c r="U40" s="23"/>
-      <c r="V40" s="24"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
+      <c r="K40" s="19"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="19"/>
+      <c r="N40" s="19"/>
+      <c r="O40" s="19"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="19"/>
+      <c r="R40" s="19"/>
+      <c r="S40" s="19"/>
+      <c r="T40" s="19"/>
+      <c r="U40" s="19"/>
+      <c r="V40" s="20"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -4110,7 +4103,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -4159,7 +4152,7 @@
         <v>72</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R42" s="1" t="s">
         <v>72</v>
@@ -4178,7 +4171,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="18"/>
+      <c r="A43" s="21"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -4225,7 +4218,7 @@
         <v>72</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R43" s="1" t="s">
         <v>72</v>
@@ -4244,7 +4237,7 @@
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="18"/>
+      <c r="A44" s="21"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -4294,7 +4287,7 @@
         <v>72</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S44" s="1" t="s">
         <v>72</v>
@@ -4310,7 +4303,7 @@
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="18"/>
+      <c r="A45" s="21"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -4376,7 +4369,7 @@
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="18"/>
+      <c r="A46" s="21"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -4442,7 +4435,7 @@
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -4510,7 +4503,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="20"/>
+      <c r="A48" s="23"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -4576,7 +4569,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="21"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -4642,28 +4635,28 @@
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="22" t="s">
+      <c r="C52" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="23"/>
-      <c r="E52" s="23"/>
-      <c r="F52" s="23"/>
-      <c r="G52" s="23"/>
-      <c r="H52" s="23"/>
-      <c r="I52" s="23"/>
-      <c r="J52" s="23"/>
-      <c r="K52" s="23"/>
-      <c r="L52" s="23"/>
-      <c r="M52" s="23"/>
-      <c r="N52" s="23"/>
-      <c r="O52" s="23"/>
-      <c r="P52" s="23"/>
-      <c r="Q52" s="23"/>
-      <c r="R52" s="23"/>
-      <c r="S52" s="23"/>
-      <c r="T52" s="23"/>
-      <c r="U52" s="23"/>
-      <c r="V52" s="24"/>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="19"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+      <c r="I52" s="19"/>
+      <c r="J52" s="19"/>
+      <c r="K52" s="19"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
+      <c r="N52" s="19"/>
+      <c r="O52" s="19"/>
+      <c r="P52" s="19"/>
+      <c r="Q52" s="19"/>
+      <c r="R52" s="19"/>
+      <c r="S52" s="19"/>
+      <c r="T52" s="19"/>
+      <c r="U52" s="19"/>
+      <c r="V52" s="20"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -4729,7 +4722,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="18" t="s">
+      <c r="A54" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
@@ -4742,19 +4735,19 @@
         <v>72</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I54" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="J54" s="1" t="s">
         <v>72</v>
@@ -4769,19 +4762,19 @@
         <v>88</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="P54" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q54" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R54" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="S54" s="1" t="s">
         <v>72</v>
@@ -4797,7 +4790,7 @@
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="18"/>
+      <c r="A55" s="21"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -4811,13 +4804,13 @@
         <v>72</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>72</v>
@@ -4838,13 +4831,13 @@
         <v>72</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="P55" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q55" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="R55" s="1" t="s">
         <v>73</v>
@@ -4853,7 +4846,7 @@
         <v>72</v>
       </c>
       <c r="T55" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="U55" s="1" t="s">
         <v>72</v>
@@ -4863,7 +4856,7 @@
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="18"/>
+      <c r="A56" s="21"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -4883,10 +4876,10 @@
         <v>72</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="J56" s="1" t="s">
         <v>72</v>
@@ -4913,23 +4906,23 @@
         <v>72</v>
       </c>
       <c r="R56" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S56" s="1" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="T56" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="U56" s="1" t="s">
         <v>72</v>
       </c>
       <c r="V56" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="18"/>
+      <c r="A57" s="21"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -4943,13 +4936,13 @@
         <v>72</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>72</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>72</v>
@@ -4967,16 +4960,16 @@
         <v>72</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="P57" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q57" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="R57" s="1" t="s">
         <v>72</v>
@@ -4991,11 +4984,11 @@
         <v>91</v>
       </c>
       <c r="V57" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="18"/>
+      <c r="A58" s="21"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -5009,7 +5002,7 @@
         <v>72</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>72</v>
@@ -5018,7 +5011,7 @@
         <v>72</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>72</v>
@@ -5027,7 +5020,7 @@
         <v>72</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="M58" s="1" t="s">
         <v>72</v>
@@ -5061,7 +5054,7 @@
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -5129,7 +5122,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="20"/>
+      <c r="A60" s="23"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -5195,7 +5188,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="21"/>
+      <c r="A61" s="24"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -5261,28 +5254,28 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="22" t="s">
+      <c r="C64" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="23"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="23"/>
-      <c r="G64" s="23"/>
-      <c r="H64" s="23"/>
-      <c r="I64" s="23"/>
-      <c r="J64" s="23"/>
-      <c r="K64" s="23"/>
-      <c r="L64" s="23"/>
-      <c r="M64" s="23"/>
-      <c r="N64" s="23"/>
-      <c r="O64" s="23"/>
-      <c r="P64" s="23"/>
-      <c r="Q64" s="23"/>
-      <c r="R64" s="23"/>
-      <c r="S64" s="23"/>
-      <c r="T64" s="23"/>
-      <c r="U64" s="23"/>
-      <c r="V64" s="24"/>
+      <c r="D64" s="19"/>
+      <c r="E64" s="19"/>
+      <c r="F64" s="19"/>
+      <c r="G64" s="19"/>
+      <c r="H64" s="19"/>
+      <c r="I64" s="19"/>
+      <c r="J64" s="19"/>
+      <c r="K64" s="19"/>
+      <c r="L64" s="19"/>
+      <c r="M64" s="19"/>
+      <c r="N64" s="19"/>
+      <c r="O64" s="19"/>
+      <c r="P64" s="19"/>
+      <c r="Q64" s="19"/>
+      <c r="R64" s="19"/>
+      <c r="S64" s="19"/>
+      <c r="T64" s="19"/>
+      <c r="U64" s="19"/>
+      <c r="V64" s="20"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -5348,7 +5341,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="18" t="s">
+      <c r="A66" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -5367,10 +5360,10 @@
         <v>72</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>72</v>
@@ -5385,10 +5378,10 @@
         <v>72</v>
       </c>
       <c r="M66" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="O66" s="1" t="s">
         <v>72</v>
@@ -5397,13 +5390,13 @@
         <v>72</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="R66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S66" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="S66" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="T66" s="1" t="s">
         <v>92</v>
@@ -5416,7 +5409,7 @@
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="18"/>
+      <c r="A67" s="21"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -5433,10 +5426,10 @@
         <v>72</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>72</v>
@@ -5466,10 +5459,10 @@
         <v>72</v>
       </c>
       <c r="R67" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S67" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="S67" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="T67" s="1" t="s">
         <v>72</v>
@@ -5482,7 +5475,7 @@
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="18"/>
+      <c r="A68" s="21"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -5502,7 +5495,7 @@
         <v>72</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>72</v>
@@ -5517,10 +5510,10 @@
         <v>72</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="O68" s="1" t="s">
         <v>72</v>
@@ -5532,23 +5525,23 @@
         <v>72</v>
       </c>
       <c r="R68" s="1" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="S68" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="T68" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U68" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="V68" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="18"/>
+      <c r="A69" s="21"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -5565,10 +5558,10 @@
         <v>72</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>72</v>
@@ -5583,7 +5576,7 @@
         <v>72</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="N69" s="1" t="s">
         <v>72</v>
@@ -5601,7 +5594,7 @@
         <v>72</v>
       </c>
       <c r="S69" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="T69" s="1" t="s">
         <v>72</v>
@@ -5614,7 +5607,7 @@
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="18"/>
+      <c r="A70" s="21"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -5637,7 +5630,7 @@
         <v>72</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="J70" s="1" t="s">
         <v>72</v>
@@ -5655,7 +5648,7 @@
         <v>72</v>
       </c>
       <c r="O70" s="1" t="s">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="P70" s="1" t="s">
         <v>72</v>
@@ -5680,7 +5673,7 @@
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="19" t="s">
+      <c r="A71" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -5748,7 +5741,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="20"/>
+      <c r="A72" s="23"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -5814,7 +5807,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="21"/>
+      <c r="A73" s="24"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -5881,16 +5874,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -5899,6 +5882,16 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix bug and remove unneccessary parts
</commit_message>
<xml_diff>
--- a/bin/excel_resources/excel_data.xlsx
+++ b/bin/excel_resources/excel_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18903091-5D99-4E82-B557-702971302EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA466B43-30DE-46CC-AB2B-2C7627C03C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="input" sheetId="1" r:id="rId1"/>
@@ -832,15 +832,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -852,6 +843,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1227,7 +1227,7 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M7" s="13" t="str">
         <f t="shared" ref="M7:M31" si="0">F$116</f>
@@ -1258,7 +1258,7 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M8" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1299,7 +1299,7 @@
         <v>85</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M9" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1329,7 +1329,7 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M10" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1360,7 +1360,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M11" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1390,7 +1390,7 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M12" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1421,7 +1421,7 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M13" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1451,7 +1451,7 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M14" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1482,7 +1482,7 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
       <c r="L15" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M15" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1513,7 +1513,7 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
       <c r="L16" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M16" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1544,7 +1544,7 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M17" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1575,7 +1575,7 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M18" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1606,7 +1606,7 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M19" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1637,7 +1637,7 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
       <c r="L20" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M20" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1667,7 +1667,7 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M21" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1697,7 +1697,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M22" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1727,7 +1727,7 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M23" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1765,7 +1765,7 @@
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M24" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1795,7 +1795,7 @@
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="L25" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M25" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1825,7 +1825,7 @@
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
       <c r="L26" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M26" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1855,7 +1855,7 @@
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
       <c r="L27" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M27" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1885,7 +1885,7 @@
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
       <c r="L28" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M28" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1915,7 +1915,7 @@
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
       <c r="L29" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M29" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1945,7 +1945,7 @@
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
       <c r="L30" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M30" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1975,7 +1975,7 @@
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
       <c r="L31" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M31" s="13" t="str">
         <f t="shared" si="0"/>
@@ -2004,8 +2004,8 @@
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
-      <c r="L32" s="1" t="s">
-        <v>22</v>
+      <c r="L32" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M32" s="1" t="s">
         <v>36</v>
@@ -2033,8 +2033,8 @@
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
-      <c r="L33" s="1" t="s">
-        <v>22</v>
+      <c r="L33" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M33" s="1" t="s">
         <v>36</v>
@@ -2062,8 +2062,8 @@
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
-      <c r="L34" s="1" t="s">
-        <v>22</v>
+      <c r="L34" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M34" s="1" t="s">
         <v>36</v>
@@ -2091,8 +2091,8 @@
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
-      <c r="L35" s="1" t="s">
-        <v>22</v>
+      <c r="L35" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M35" s="1" t="s">
         <v>36</v>
@@ -2120,8 +2120,8 @@
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
-      <c r="L36" s="1" t="s">
-        <v>22</v>
+      <c r="L36" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M36" s="1" t="s">
         <v>36</v>
@@ -2149,8 +2149,8 @@
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
-      <c r="L37" s="1" t="s">
-        <v>22</v>
+      <c r="L37" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M37" s="1" t="s">
         <v>36</v>
@@ -2178,8 +2178,8 @@
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
-      <c r="L38" s="1" t="s">
-        <v>22</v>
+      <c r="L38" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M38" s="1" t="s">
         <v>36</v>
@@ -2207,8 +2207,8 @@
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
-      <c r="L39" s="1" t="s">
-        <v>22</v>
+      <c r="L39" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M39" s="1" t="s">
         <v>36</v>
@@ -2236,8 +2236,8 @@
       <c r="I40" s="1"/>
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
-      <c r="L40" s="1" t="s">
-        <v>22</v>
+      <c r="L40" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M40" s="1" t="s">
         <v>36</v>
@@ -2265,8 +2265,8 @@
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
       <c r="K41" s="1"/>
-      <c r="L41" s="1" t="s">
-        <v>22</v>
+      <c r="L41" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M41" s="1" t="s">
         <v>36</v>
@@ -2294,8 +2294,8 @@
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
-      <c r="L42" s="1" t="s">
-        <v>22</v>
+      <c r="L42" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M42" s="1" t="s">
         <v>36</v>
@@ -2323,8 +2323,8 @@
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
-      <c r="L43" s="1" t="s">
-        <v>22</v>
+      <c r="L43" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M43" s="1" t="s">
         <v>36</v>
@@ -2352,8 +2352,8 @@
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
-      <c r="L44" s="1" t="s">
-        <v>22</v>
+      <c r="L44" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M44" s="1" t="s">
         <v>36</v>
@@ -2381,8 +2381,8 @@
       <c r="I45" s="1"/>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
-      <c r="L45" s="1" t="s">
-        <v>22</v>
+      <c r="L45" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M45" s="1" t="s">
         <v>36</v>
@@ -2410,8 +2410,8 @@
       <c r="I46" s="1"/>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
-      <c r="L46" s="1" t="s">
-        <v>22</v>
+      <c r="L46" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M46" s="1" t="s">
         <v>36</v>
@@ -2439,8 +2439,8 @@
       <c r="I47" s="1"/>
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
-      <c r="L47" s="1" t="s">
-        <v>22</v>
+      <c r="L47" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M47" s="1" t="s">
         <v>36</v>
@@ -2468,8 +2468,8 @@
       <c r="I48" s="1"/>
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
-      <c r="L48" s="1" t="s">
-        <v>22</v>
+      <c r="L48" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M48" s="1" t="s">
         <v>36</v>
@@ -2497,8 +2497,8 @@
       <c r="I49" s="1"/>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
-      <c r="L49" s="1" t="s">
-        <v>22</v>
+      <c r="L49" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M49" s="1" t="s">
         <v>36</v>
@@ -2526,8 +2526,8 @@
       <c r="I50" s="1"/>
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
-      <c r="L50" s="1" t="s">
-        <v>22</v>
+      <c r="L50" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M50" s="1" t="s">
         <v>36</v>
@@ -2555,8 +2555,8 @@
       <c r="I51" s="1"/>
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
-      <c r="L51" s="1" t="s">
-        <v>22</v>
+      <c r="L51" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M51" s="1" t="s">
         <v>36</v>
@@ -2584,8 +2584,8 @@
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
-      <c r="L52" s="1" t="s">
-        <v>22</v>
+      <c r="L52" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M52" s="1" t="s">
         <v>36</v>
@@ -2613,8 +2613,8 @@
       <c r="I53" s="1"/>
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
-      <c r="L53" s="1" t="s">
-        <v>22</v>
+      <c r="L53" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M53" s="1" t="s">
         <v>36</v>
@@ -2642,8 +2642,8 @@
       <c r="I54" s="1"/>
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
-      <c r="L54" s="1" t="s">
-        <v>22</v>
+      <c r="L54" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M54" s="1" t="s">
         <v>36</v>
@@ -2671,8 +2671,8 @@
       <c r="I55" s="1"/>
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
-      <c r="L55" s="1" t="s">
-        <v>22</v>
+      <c r="L55" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M55" s="1" t="s">
         <v>36</v>
@@ -2700,8 +2700,8 @@
       <c r="I56" s="1"/>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
-      <c r="L56" s="1" t="s">
-        <v>22</v>
+      <c r="L56" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M56" s="1" t="s">
         <v>36</v>
@@ -2729,8 +2729,8 @@
       <c r="I57" s="1"/>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
-      <c r="L57" s="1" t="s">
-        <v>22</v>
+      <c r="L57" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M57" s="1" t="s">
         <v>36</v>
@@ -2758,8 +2758,8 @@
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
-      <c r="L58" s="1" t="s">
-        <v>22</v>
+      <c r="L58" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M58" s="1" t="s">
         <v>36</v>
@@ -2787,8 +2787,8 @@
       <c r="I59" s="1"/>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
-      <c r="L59" s="1" t="s">
-        <v>22</v>
+      <c r="L59" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M59" s="1" t="s">
         <v>36</v>
@@ -2816,8 +2816,8 @@
       <c r="I60" s="1"/>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
-      <c r="L60" s="1" t="s">
-        <v>22</v>
+      <c r="L60" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M60" s="1" t="s">
         <v>36</v>
@@ -2845,8 +2845,8 @@
       <c r="I61" s="1"/>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
-      <c r="L61" s="1" t="s">
-        <v>22</v>
+      <c r="L61" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M61" s="1" t="s">
         <v>36</v>
@@ -2874,8 +2874,8 @@
       <c r="I62" s="1"/>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
-      <c r="L62" s="1" t="s">
-        <v>24</v>
+      <c r="L62" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M62" s="1" t="s">
         <v>35</v>
@@ -2892,7 +2892,7 @@
         <v>61</v>
       </c>
       <c r="D63" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E63" s="1">
         <v>70</v>
@@ -2903,8 +2903,8 @@
       <c r="I63" s="1"/>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
-      <c r="L63" s="1" t="s">
-        <v>24</v>
+      <c r="L63" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M63" s="1" t="s">
         <v>35</v>
@@ -2921,7 +2921,7 @@
         <v>61</v>
       </c>
       <c r="D64" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E64" s="1">
         <v>70</v>
@@ -2932,8 +2932,8 @@
       <c r="I64" s="1"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
-      <c r="L64" s="1" t="s">
-        <v>24</v>
+      <c r="L64" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M64" s="1" t="s">
         <v>35</v>
@@ -2950,7 +2950,7 @@
         <v>61</v>
       </c>
       <c r="D65" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E65" s="1">
         <v>50</v>
@@ -2961,8 +2961,8 @@
       <c r="I65" s="1"/>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
-      <c r="L65" s="1" t="s">
-        <v>24</v>
+      <c r="L65" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M65" s="1" t="s">
         <v>35</v>
@@ -3637,7 +3637,7 @@
         <v>21</v>
       </c>
       <c r="D123" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E123" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3659,7 +3659,7 @@
         <v>21</v>
       </c>
       <c r="D124" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E124" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3703,7 +3703,7 @@
         <v>21</v>
       </c>
       <c r="D126" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E126" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3725,7 +3725,7 @@
         <v>21</v>
       </c>
       <c r="D127" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E127" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3747,7 +3747,7 @@
         <v>21</v>
       </c>
       <c r="D128" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E128" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3769,7 +3769,7 @@
         <v>21</v>
       </c>
       <c r="D129" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E129" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3837,7 +3837,7 @@
         <v>21</v>
       </c>
       <c r="D132" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E132" s="2" t="b">
         <v>0</v>
@@ -4000,28 +4000,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="20"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20"/>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="21"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="25"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -4087,7 +4087,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -4145,22 +4145,22 @@
         <v>166</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>155</v>
+        <v>179</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="V6" s="1" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="22"/>
+      <c r="A7" s="19"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>152</v>
@@ -4172,10 +4172,10 @@
         <v>154</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>157</v>
@@ -4187,148 +4187,148 @@
         <v>160</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>163</v>
+        <v>72</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="O7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q7" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="P7" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="R7" s="1" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>166</v>
       </c>
       <c r="T7" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="V7" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="U7" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>162</v>
-      </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="22"/>
+      <c r="A8" s="19"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>151</v>
+        <v>179</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>156</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>172</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="L8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="S8" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="T8" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="V8" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="U8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>165</v>
-      </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="22"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>170</v>
+        <v>72</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>181</v>
+        <v>72</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>153</v>
+        <v>72</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>169</v>
+        <v>72</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>178</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>173</v>
+        <v>72</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>154</v>
+        <v>72</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>151</v>
+        <v>72</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>72</v>
@@ -4337,31 +4337,31 @@
         <v>155</v>
       </c>
       <c r="R9" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="S9" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="S9" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="T9" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="U9" s="1" t="s">
         <v>72</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="22"/>
+      <c r="A10" s="19"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>174</v>
+        <v>72</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>72</v>
@@ -4370,47 +4370,47 @@
         <v>72</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>153</v>
+        <v>72</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>196</v>
+        <v>72</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>171</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>173</v>
+        <v>72</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>154</v>
+        <v>72</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="T10" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="R10" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="S10" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>179</v>
-      </c>
       <c r="U10" s="1" t="s">
         <v>72</v>
       </c>
@@ -4419,51 +4419,51 @@
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
         <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>72</v>
+        <v>184</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>72</v>
+        <v>189</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>72</v>
+        <v>190</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>185</v>
       </c>
       <c r="K11" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O11" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="L11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>197</v>
-      </c>
       <c r="P11" s="1" t="s">
         <v>72</v>
       </c>
@@ -4487,24 +4487,24 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="24"/>
+      <c r="A12" s="21"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="E12" s="1" t="s">
-        <v>188</v>
+        <v>72</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>72</v>
+        <v>189</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>72</v>
+        <v>190</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>72</v>
@@ -4513,13 +4513,13 @@
         <v>72</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>191</v>
+        <v>72</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>192</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>72</v>
+        <v>197</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>72</v>
@@ -4553,7 +4553,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="25"/>
+      <c r="A13" s="22"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -4567,7 +4567,7 @@
         <v>72</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>72</v>
+        <v>190</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>72</v>
@@ -4619,28 +4619,28 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="20"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="20"/>
-      <c r="Q16" s="20"/>
-      <c r="R16" s="20"/>
-      <c r="S16" s="20"/>
-      <c r="T16" s="20"/>
-      <c r="U16" s="20"/>
-      <c r="V16" s="21"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+      <c r="O16" s="24"/>
+      <c r="P16" s="24"/>
+      <c r="Q16" s="24"/>
+      <c r="R16" s="24"/>
+      <c r="S16" s="24"/>
+      <c r="T16" s="24"/>
+      <c r="U16" s="24"/>
+      <c r="V16" s="25"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -4706,14 +4706,14 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>152</v>
@@ -4722,191 +4722,191 @@
         <v>153</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>157</v>
       </c>
       <c r="J18" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="L18" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="L18" s="1" t="s">
-        <v>169</v>
-      </c>
       <c r="M18" s="1" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="O18" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q18" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="P18" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>176</v>
-      </c>
       <c r="R18" s="1" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="S18" s="1" t="s">
         <v>166</v>
       </c>
       <c r="T18" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="V18" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="22"/>
+      <c r="A19" s="19"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="I19" s="1" t="s">
-        <v>72</v>
+        <v>157</v>
       </c>
       <c r="J19" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K19" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="L19" s="1" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>159</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>72</v>
+        <v>162</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="V19" s="1" t="s">
-        <v>72</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="22"/>
+      <c r="A20" s="19"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>175</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="J20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K20" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="K20" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="L20" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>72</v>
+        <v>154</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>72</v>
+        <v>174</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>72</v>
+        <v>157</v>
       </c>
       <c r="V20" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="22"/>
+      <c r="A21" s="19"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -4923,19 +4923,19 @@
         <v>72</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>72</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>72</v>
+        <v>178</v>
       </c>
       <c r="L21" s="1" t="s">
         <v>72</v>
@@ -4944,7 +4944,7 @@
         <v>72</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>72</v>
@@ -4953,26 +4953,26 @@
         <v>72</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>72</v>
+        <v>177</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>72</v>
+        <v>175</v>
       </c>
       <c r="T21" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="V21" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="22"/>
+      <c r="A22" s="19"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -5022,7 +5022,7 @@
         <v>72</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>72</v>
+        <v>177</v>
       </c>
       <c r="S22" s="1" t="s">
         <v>72</v>
@@ -5038,41 +5038,41 @@
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
         <v>6</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>72</v>
+        <v>193</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>72</v>
+        <v>188</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>72</v>
+        <v>183</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>72</v>
+        <v>187</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>72</v>
+        <v>184</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>72</v>
+        <v>189</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>72</v>
+        <v>191</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="M23" s="1" t="s">
         <v>186</v>
@@ -5106,7 +5106,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="24"/>
+      <c r="A24" s="21"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -5117,7 +5117,7 @@
         <v>72</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>72</v>
+        <v>188</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>72</v>
@@ -5141,7 +5141,7 @@
         <v>72</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>72</v>
+        <v>197</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>72</v>
@@ -5172,7 +5172,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="25"/>
+      <c r="A25" s="22"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -5238,28 +5238,28 @@
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
-      <c r="M28" s="20"/>
-      <c r="N28" s="20"/>
-      <c r="O28" s="20"/>
-      <c r="P28" s="20"/>
-      <c r="Q28" s="20"/>
-      <c r="R28" s="20"/>
-      <c r="S28" s="20"/>
-      <c r="T28" s="20"/>
-      <c r="U28" s="20"/>
-      <c r="V28" s="21"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
+      <c r="N28" s="24"/>
+      <c r="O28" s="24"/>
+      <c r="P28" s="24"/>
+      <c r="Q28" s="24"/>
+      <c r="R28" s="24"/>
+      <c r="S28" s="24"/>
+      <c r="T28" s="24"/>
+      <c r="U28" s="24"/>
+      <c r="V28" s="25"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -5325,7 +5325,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -5335,7 +5335,7 @@
         <v>170</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>179</v>
+        <v>151</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>152</v>
@@ -5347,53 +5347,53 @@
         <v>175</v>
       </c>
       <c r="H30" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I30" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I30" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="J30" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>154</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="M30" s="1" t="s">
         <v>159</v>
       </c>
       <c r="N30" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="O30" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="O30" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="P30" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q30" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="R30" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="R30" s="1" t="s">
+      <c r="S30" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>155</v>
       </c>
       <c r="T30" s="1" t="s">
         <v>157</v>
       </c>
       <c r="U30" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V30" s="1" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="22"/>
+      <c r="A31" s="19"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -5401,7 +5401,7 @@
         <v>174</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>152</v>
@@ -5410,199 +5410,199 @@
         <v>153</v>
       </c>
       <c r="G31" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="H31" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="H31" s="1" t="s">
-        <v>196</v>
-      </c>
       <c r="I31" s="1" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>154</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="P31" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q31" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="R31" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="R31" s="1" t="s">
-        <v>175</v>
-      </c>
       <c r="S31" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="T31" s="1" t="s">
         <v>157</v>
       </c>
       <c r="U31" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V31" s="1" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="22"/>
+      <c r="A32" s="19"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>167</v>
+        <v>195</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="F32" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I32" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>161</v>
       </c>
       <c r="K32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="R32" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="S32" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="T32" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="L32" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="M32" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="N32" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q32" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="R32" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="S32" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="T32" s="1" t="s">
+      <c r="U32" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="U32" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="V32" s="1" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="22"/>
+      <c r="A33" s="19"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>177</v>
+        <v>72</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>173</v>
+        <v>195</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="G33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M33" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="G33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H33" s="1" t="s">
+      <c r="N33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q33" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="R33" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="S33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U33" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="I33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="K33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L33" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="M33" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q33" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="R33" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="S33" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="T33" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="U33" s="1" t="s">
-        <v>179</v>
-      </c>
       <c r="V33" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="22"/>
+      <c r="A34" s="19"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>167</v>
+        <v>72</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>72</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>174</v>
+        <v>72</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>72</v>
@@ -5611,19 +5611,19 @@
         <v>72</v>
       </c>
       <c r="H34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I34" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="K34" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>169</v>
+        <v>72</v>
       </c>
       <c r="M34" s="1" t="s">
         <v>72</v>
@@ -5638,11 +5638,11 @@
         <v>72</v>
       </c>
       <c r="Q34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R34" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="R34" s="1" t="s">
-        <v>158</v>
-      </c>
       <c r="S34" s="1" t="s">
         <v>72</v>
       </c>
@@ -5657,7 +5657,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="23" t="s">
+      <c r="A35" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -5667,29 +5667,29 @@
         <v>72</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>193</v>
+        <v>72</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>72</v>
       </c>
       <c r="F35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="K35" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="L35" s="1" t="s">
         <v>72</v>
       </c>
@@ -5697,10 +5697,10 @@
         <v>72</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>72</v>
+        <v>186</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>72</v>
+        <v>197</v>
       </c>
       <c r="P35" s="1" t="s">
         <v>72</v>
@@ -5725,7 +5725,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="24"/>
+      <c r="A36" s="21"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -5733,7 +5733,7 @@
         <v>72</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>188</v>
+        <v>72</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>72</v>
@@ -5763,7 +5763,7 @@
         <v>72</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>72</v>
+        <v>197</v>
       </c>
       <c r="O36" s="1" t="s">
         <v>72</v>
@@ -5791,7 +5791,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="25"/>
+      <c r="A37" s="22"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -5799,7 +5799,7 @@
         <v>72</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>182</v>
+        <v>72</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>72</v>
@@ -5857,28 +5857,28 @@
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="19" t="s">
+      <c r="C40" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
-      <c r="L40" s="20"/>
-      <c r="M40" s="20"/>
-      <c r="N40" s="20"/>
-      <c r="O40" s="20"/>
-      <c r="P40" s="20"/>
-      <c r="Q40" s="20"/>
-      <c r="R40" s="20"/>
-      <c r="S40" s="20"/>
-      <c r="T40" s="20"/>
-      <c r="U40" s="20"/>
-      <c r="V40" s="21"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="24"/>
+      <c r="J40" s="24"/>
+      <c r="K40" s="24"/>
+      <c r="L40" s="24"/>
+      <c r="M40" s="24"/>
+      <c r="N40" s="24"/>
+      <c r="O40" s="24"/>
+      <c r="P40" s="24"/>
+      <c r="Q40" s="24"/>
+      <c r="R40" s="24"/>
+      <c r="S40" s="24"/>
+      <c r="T40" s="24"/>
+      <c r="U40" s="24"/>
+      <c r="V40" s="25"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -5944,26 +5944,26 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="22" t="s">
+      <c r="A42" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
         <v>1</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>170</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>181</v>
+        <v>155</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>171</v>
@@ -5972,19 +5972,19 @@
         <v>156</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>176</v>
+        <v>154</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>72</v>
+        <v>151</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="O42" s="1" t="s">
         <v>162</v>
@@ -5996,64 +5996,64 @@
         <v>158</v>
       </c>
       <c r="R42" s="1" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="S42" s="1" t="s">
         <v>165</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>178</v>
+        <v>157</v>
       </c>
       <c r="U42" s="1" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="V42" s="1" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="22"/>
+      <c r="A43" s="19"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>174</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>72</v>
+        <v>181</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>196</v>
+        <v>155</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="K43" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="M43" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="L43" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M43" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="N43" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="P43" s="1" t="s">
         <v>72</v>
@@ -6062,40 +6062,40 @@
         <v>158</v>
       </c>
       <c r="R43" s="1" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="T43" s="1" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="U43" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="V43" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="V43" s="1" t="s">
-        <v>165</v>
-      </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="22"/>
+      <c r="A44" s="19"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>72</v>
+        <v>175</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="H44" s="1" t="s">
         <v>72</v>
@@ -6104,16 +6104,16 @@
         <v>72</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>72</v>
+        <v>161</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>72</v>
+        <v>154</v>
       </c>
       <c r="N44" s="1" t="s">
         <v>72</v>
@@ -6125,26 +6125,26 @@
         <v>72</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="T44" s="1" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="U44" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="V44" s="1" t="s">
-        <v>72</v>
+        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="22"/>
+      <c r="A45" s="19"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -6155,13 +6155,13 @@
         <v>72</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>72</v>
+        <v>181</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="H45" s="1" t="s">
         <v>72</v>
@@ -6170,16 +6170,16 @@
         <v>72</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="L45" s="1" t="s">
         <v>72</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>72</v>
@@ -6191,26 +6191,26 @@
         <v>72</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>72</v>
+        <v>174</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="T45" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U45" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="V45" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="22"/>
+      <c r="A46" s="19"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -6236,7 +6236,7 @@
         <v>72</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="K46" s="1" t="s">
         <v>72</v>
@@ -6269,14 +6269,14 @@
         <v>72</v>
       </c>
       <c r="U46" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="V46" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="23" t="s">
+      <c r="A47" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -6289,7 +6289,7 @@
         <v>72</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>193</v>
+        <v>72</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>72</v>
@@ -6316,10 +6316,10 @@
         <v>72</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>72</v>
+        <v>186</v>
       </c>
       <c r="P47" s="1" t="s">
         <v>72</v>
@@ -6344,7 +6344,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="24"/>
+      <c r="A48" s="21"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -6385,7 +6385,7 @@
         <v>72</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>72</v>
+        <v>198</v>
       </c>
       <c r="P48" s="1" t="s">
         <v>72</v>
@@ -6410,7 +6410,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="25"/>
+      <c r="A49" s="22"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -6476,28 +6476,28 @@
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="19" t="s">
+      <c r="C52" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="20"/>
-      <c r="E52" s="20"/>
-      <c r="F52" s="20"/>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20"/>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20"/>
-      <c r="L52" s="20"/>
-      <c r="M52" s="20"/>
-      <c r="N52" s="20"/>
-      <c r="O52" s="20"/>
-      <c r="P52" s="20"/>
-      <c r="Q52" s="20"/>
-      <c r="R52" s="20"/>
-      <c r="S52" s="20"/>
-      <c r="T52" s="20"/>
-      <c r="U52" s="20"/>
-      <c r="V52" s="21"/>
+      <c r="D52" s="24"/>
+      <c r="E52" s="24"/>
+      <c r="F52" s="24"/>
+      <c r="G52" s="24"/>
+      <c r="H52" s="24"/>
+      <c r="I52" s="24"/>
+      <c r="J52" s="24"/>
+      <c r="K52" s="24"/>
+      <c r="L52" s="24"/>
+      <c r="M52" s="24"/>
+      <c r="N52" s="24"/>
+      <c r="O52" s="24"/>
+      <c r="P52" s="24"/>
+      <c r="Q52" s="24"/>
+      <c r="R52" s="24"/>
+      <c r="S52" s="24"/>
+      <c r="T52" s="24"/>
+      <c r="U52" s="24"/>
+      <c r="V52" s="25"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -6563,92 +6563,92 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="22" t="s">
+      <c r="A54" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
         <v>1</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D54" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M54" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N54" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="L54" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="N54" s="1" t="s">
+      <c r="O54" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="O54" s="1" t="s">
+      <c r="P54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q54" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="P54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q54" s="1" t="s">
+      <c r="R54" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="R54" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="S54" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="T54" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="T54" s="1" t="s">
+      <c r="U54" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="U54" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="V54" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="22"/>
+      <c r="A55" s="19"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>72</v>
+        <v>174</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>196</v>
+        <v>152</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>181</v>
+        <v>153</v>
       </c>
       <c r="H55" s="1" t="s">
         <v>155</v>
@@ -6657,85 +6657,85 @@
         <v>166</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="L55" s="1" t="s">
         <v>154</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="N55" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="O55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q55" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="R55" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="S55" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="O55" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P55" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q55" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="R55" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="S55" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="T55" s="1" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="U55" s="1" t="s">
         <v>165</v>
       </c>
       <c r="V55" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="22"/>
+      <c r="A56" s="19"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>173</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="F56" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="G56" s="1" t="s">
-        <v>152</v>
+        <v>196</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>178</v>
+        <v>159</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="O56" s="1" t="s">
         <v>72</v>
@@ -6744,92 +6744,92 @@
         <v>72</v>
       </c>
       <c r="Q56" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="R56" s="1" t="s">
         <v>161</v>
       </c>
       <c r="S56" s="1" t="s">
-        <v>164</v>
+        <v>72</v>
       </c>
       <c r="T56" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U56" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="V56" s="1" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="22"/>
+      <c r="A57" s="19"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>72</v>
+        <v>195</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>167</v>
+        <v>72</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>174</v>
+        <v>72</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>196</v>
+        <v>72</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="I57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q57" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="R57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T57" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="J57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L57" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="M57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N57" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="O57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="R57" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="S57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T57" s="1" t="s">
-        <v>180</v>
-      </c>
       <c r="U57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="V57" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="V57" s="1" t="s">
-        <v>177</v>
-      </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="22"/>
+      <c r="A58" s="19"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -6846,13 +6846,13 @@
         <v>72</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>152</v>
+        <v>72</v>
       </c>
       <c r="H58" s="1" t="s">
         <v>72</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>72</v>
@@ -6867,7 +6867,7 @@
         <v>72</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>154</v>
+        <v>72</v>
       </c>
       <c r="O58" s="1" t="s">
         <v>72</v>
@@ -6879,30 +6879,30 @@
         <v>72</v>
       </c>
       <c r="R58" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="S58" s="1" t="s">
         <v>72</v>
       </c>
       <c r="T58" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="U58" s="1" t="s">
-        <v>166</v>
+        <v>72</v>
       </c>
       <c r="V58" s="1" t="s">
-        <v>167</v>
+        <v>72</v>
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="23" t="s">
+      <c r="A59" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
         <v>6</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>188</v>
+        <v>72</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>72</v>
@@ -6911,34 +6911,34 @@
         <v>72</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>184</v>
+        <v>72</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>189</v>
+        <v>72</v>
       </c>
       <c r="H59" s="1" t="s">
         <v>72</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>200</v>
+        <v>72</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>199</v>
+        <v>72</v>
       </c>
       <c r="K59" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>186</v>
+        <v>72</v>
       </c>
       <c r="M59" s="1" t="s">
         <v>187</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="O59" s="1" t="s">
-        <v>198</v>
+        <v>72</v>
       </c>
       <c r="P59" s="1" t="s">
         <v>72</v>
@@ -6963,7 +6963,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="24"/>
+      <c r="A60" s="21"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -6977,10 +6977,10 @@
         <v>72</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>189</v>
+        <v>72</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="H60" s="1" t="s">
         <v>72</v>
@@ -6998,7 +6998,7 @@
         <v>72</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>197</v>
+        <v>72</v>
       </c>
       <c r="N60" s="1" t="s">
         <v>72</v>
@@ -7029,7 +7029,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="25"/>
+      <c r="A61" s="22"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -7043,7 +7043,7 @@
         <v>72</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>72</v>
@@ -7064,7 +7064,7 @@
         <v>72</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="N61" s="1" t="s">
         <v>72</v>
@@ -7095,28 +7095,28 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="19" t="s">
+      <c r="C64" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="20"/>
-      <c r="E64" s="20"/>
-      <c r="F64" s="20"/>
-      <c r="G64" s="20"/>
-      <c r="H64" s="20"/>
-      <c r="I64" s="20"/>
-      <c r="J64" s="20"/>
-      <c r="K64" s="20"/>
-      <c r="L64" s="20"/>
-      <c r="M64" s="20"/>
-      <c r="N64" s="20"/>
-      <c r="O64" s="20"/>
-      <c r="P64" s="20"/>
-      <c r="Q64" s="20"/>
-      <c r="R64" s="20"/>
-      <c r="S64" s="20"/>
-      <c r="T64" s="20"/>
-      <c r="U64" s="20"/>
-      <c r="V64" s="21"/>
+      <c r="D64" s="24"/>
+      <c r="E64" s="24"/>
+      <c r="F64" s="24"/>
+      <c r="G64" s="24"/>
+      <c r="H64" s="24"/>
+      <c r="I64" s="24"/>
+      <c r="J64" s="24"/>
+      <c r="K64" s="24"/>
+      <c r="L64" s="24"/>
+      <c r="M64" s="24"/>
+      <c r="N64" s="24"/>
+      <c r="O64" s="24"/>
+      <c r="P64" s="24"/>
+      <c r="Q64" s="24"/>
+      <c r="R64" s="24"/>
+      <c r="S64" s="24"/>
+      <c r="T64" s="24"/>
+      <c r="U64" s="24"/>
+      <c r="V64" s="25"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -7182,20 +7182,20 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="22" t="s">
+      <c r="A66" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
         <v>1</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>152</v>
@@ -7204,25 +7204,25 @@
         <v>153</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>196</v>
+        <v>155</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="J66" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="K66" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="L66" s="1" t="s">
         <v>154</v>
       </c>
       <c r="M66" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N66" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="N66" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="O66" s="1" t="s">
         <v>169</v>
@@ -7231,7 +7231,7 @@
         <v>72</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="R66" s="1" t="s">
         <v>158</v>
@@ -7240,17 +7240,17 @@
         <v>162</v>
       </c>
       <c r="T66" s="1" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="U66" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="V66" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="22"/>
+      <c r="A67" s="19"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -7258,10 +7258,10 @@
         <v>173</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>195</v>
+        <v>174</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>152</v>
@@ -7270,67 +7270,67 @@
         <v>153</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="J67" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="L67" s="1" t="s">
         <v>154</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N67" s="1" t="s">
         <v>171</v>
       </c>
       <c r="O67" s="1" t="s">
-        <v>151</v>
+        <v>72</v>
       </c>
       <c r="P67" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q67" s="1" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="R67" s="1" t="s">
         <v>158</v>
       </c>
       <c r="S67" s="1" t="s">
-        <v>176</v>
+        <v>155</v>
       </c>
       <c r="T67" s="1" t="s">
         <v>166</v>
       </c>
       <c r="U67" s="1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="V67" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="22"/>
+      <c r="A68" s="19"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>195</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>196</v>
@@ -7339,50 +7339,50 @@
         <v>72</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="K68" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>72</v>
+        <v>161</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
       <c r="P68" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q68" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="R68" s="1" t="s">
         <v>155</v>
       </c>
       <c r="S68" s="1" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="T68" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U68" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="V68" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="U68" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="V68" s="1" t="s">
-        <v>177</v>
-      </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="22"/>
+      <c r="A69" s="19"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -7390,22 +7390,22 @@
         <v>72</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>195</v>
+        <v>72</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="H69" s="1" t="s">
         <v>72</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="J69" s="1" t="s">
         <v>72</v>
@@ -7417,38 +7417,38 @@
         <v>72</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>151</v>
+        <v>72</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
       <c r="P69" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q69" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R69" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S69" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T69" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U69" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="R69" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="S69" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="T69" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="U69" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="V69" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="22"/>
+      <c r="A70" s="19"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -7459,10 +7459,10 @@
         <v>72</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>195</v>
+        <v>72</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>72</v>
@@ -7471,7 +7471,7 @@
         <v>72</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="J70" s="1" t="s">
         <v>72</v>
@@ -7483,38 +7483,38 @@
         <v>72</v>
       </c>
       <c r="M70" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="N70" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O70" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
       <c r="P70" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q70" s="1" t="s">
-        <v>177</v>
+        <v>72</v>
       </c>
       <c r="R70" s="1" t="s">
         <v>72</v>
       </c>
       <c r="S70" s="1" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="T70" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="U70" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="V70" s="1" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="23" t="s">
+      <c r="A71" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -7536,7 +7536,7 @@
         <v>72</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>184</v>
+        <v>72</v>
       </c>
       <c r="I71" s="1" t="s">
         <v>72</v>
@@ -7545,10 +7545,10 @@
         <v>72</v>
       </c>
       <c r="K71" s="1" t="s">
-        <v>191</v>
+        <v>72</v>
       </c>
       <c r="L71" s="1" t="s">
-        <v>197</v>
+        <v>72</v>
       </c>
       <c r="M71" s="1" t="s">
         <v>72</v>
@@ -7557,7 +7557,7 @@
         <v>187</v>
       </c>
       <c r="O71" s="1" t="s">
-        <v>186</v>
+        <v>72</v>
       </c>
       <c r="P71" s="1" t="s">
         <v>72</v>
@@ -7582,7 +7582,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="24"/>
+      <c r="A72" s="21"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -7602,7 +7602,7 @@
         <v>72</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>189</v>
+        <v>72</v>
       </c>
       <c r="I72" s="1" t="s">
         <v>72</v>
@@ -7614,16 +7614,16 @@
         <v>72</v>
       </c>
       <c r="L72" s="1" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="M72" s="1" t="s">
         <v>72</v>
       </c>
       <c r="N72" s="1" t="s">
-        <v>186</v>
+        <v>72</v>
       </c>
       <c r="O72" s="1" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="P72" s="1" t="s">
         <v>72</v>
@@ -7648,7 +7648,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="25"/>
+      <c r="A73" s="22"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -7686,7 +7686,7 @@
         <v>72</v>
       </c>
       <c r="N73" s="1" t="s">
-        <v>197</v>
+        <v>72</v>
       </c>
       <c r="O73" s="1" t="s">
         <v>72</v>
@@ -7715,6 +7715,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -7723,16 +7733,6 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactoring + prioritize arrange main course first
</commit_message>
<xml_diff>
--- a/bin/excel_resources/excel_data.xlsx
+++ b/bin/excel_resources/excel_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA466B43-30DE-46CC-AB2B-2C7627C03C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08FA4CB6-FAF4-4EE1-A3C6-1261EAAC1D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3371" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10071" uniqueCount="190">
   <si>
     <t>10A1</t>
   </si>
@@ -457,33 +457,6 @@
     <t>10A4,10A5,10A6,10A7,11B1,11B2,11B4,11B5</t>
   </si>
   <si>
-    <t>Hoàng Thanh Đô</t>
-  </si>
-  <si>
-    <t>10A1,10A2,10A3,10A4,10A5,10A6,10A7,11B1,11B2,11B3,11B4,11B5,11B6, 12C1,12C2,12C3,12C4,12C5,12C6</t>
-  </si>
-  <si>
-    <t>Nguyễn Đình Phúc</t>
-  </si>
-  <si>
-    <t>11B1,11B2,12C1,12C2,12C3,12C4,12C5,12C6</t>
-  </si>
-  <si>
-    <t>Hoàng Thanh Quang</t>
-  </si>
-  <si>
-    <t>10A1,10A2,10A3,10A4,10A5,11B3,11B4,11B5,11B6</t>
-  </si>
-  <si>
-    <t>Ngô Thị Hà Chang</t>
-  </si>
-  <si>
-    <t>10A6,10A7</t>
-  </si>
-  <si>
-    <t>Hoàng Thanh Quang-TD</t>
-  </si>
-  <si>
     <t>Củng Thị Trường-Anh</t>
   </si>
   <si>
@@ -544,9 +517,6 @@
     <t>Phạm Văn Đoàn-Tin</t>
   </si>
   <si>
-    <t>Ngô Thị Hà Chang-TD</t>
-  </si>
-  <si>
     <t>Vi Văn Tình-Văn</t>
   </si>
   <si>
@@ -554,9 +524,6 @@
   </si>
   <si>
     <t>Nguyễn Thị Hằng-Sử</t>
-  </si>
-  <si>
-    <t>Nguyễn Đình Phúc-TD</t>
   </si>
   <si>
     <t>Tạ Thanh Hải-Anh</t>
@@ -2853,120 +2820,64 @@
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A62" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D62" s="1">
-        <v>1</v>
-      </c>
-      <c r="E62" s="1">
-        <v>35</v>
-      </c>
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+      <c r="C62" s="1"/>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
       <c r="H62" s="1"/>
       <c r="I62" s="1"/>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
-      <c r="L62" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="M62" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="L62" s="13"/>
+      <c r="M62" s="1"/>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A63" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D63" s="1">
-        <v>1</v>
-      </c>
-      <c r="E63" s="1">
-        <v>70</v>
-      </c>
+      <c r="A63" s="1"/>
+      <c r="B63" s="1"/>
+      <c r="C63" s="1"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
       <c r="H63" s="1"/>
       <c r="I63" s="1"/>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
-      <c r="L63" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="M63" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="L63" s="13"/>
+      <c r="M63" s="1"/>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A64" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D64" s="1">
-        <v>1</v>
-      </c>
-      <c r="E64" s="1">
-        <v>70</v>
-      </c>
+      <c r="A64" s="1"/>
+      <c r="B64" s="1"/>
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
       <c r="I64" s="1"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
-      <c r="L64" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="M64" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="L64" s="13"/>
+      <c r="M64" s="1"/>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A65" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D65" s="1">
-        <v>1</v>
-      </c>
-      <c r="E65" s="1">
-        <v>50</v>
-      </c>
+      <c r="A65" s="1"/>
+      <c r="B65" s="1"/>
+      <c r="C65" s="1"/>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1"/>
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
-      <c r="L65" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="M65" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="L65" s="13"/>
+      <c r="M65" s="1"/>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A66" s="1"/>
@@ -4094,64 +4005,64 @@
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="L6" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="R6" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="I6" s="1" t="s">
+      <c r="S6" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K6" s="1" t="s">
+      <c r="T6" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="V6" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
@@ -4160,64 +4071,64 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q7" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H7" s="1" t="s">
+      <c r="R7" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="V7" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="S7" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
@@ -4226,64 +4137,64 @@
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>72</v>
+        <v>161</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="U8" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>157</v>
-      </c>
       <c r="V8" s="1" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
@@ -4295,28 +4206,28 @@
         <v>72</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>72</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>196</v>
+        <v>146</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>72</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>178</v>
+        <v>162</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>72</v>
@@ -4325,7 +4236,7 @@
         <v>72</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>72</v>
@@ -4334,22 +4245,22 @@
         <v>72</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>177</v>
+        <v>72</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
@@ -4382,7 +4293,7 @@
         <v>72</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="L10" s="1" t="s">
         <v>72</v>
@@ -4403,19 +4314,19 @@
         <v>72</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>177</v>
+        <v>72</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
       <c r="U10" s="1" t="s">
         <v>72</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
@@ -4426,43 +4337,43 @@
         <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>193</v>
+        <v>172</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>200</v>
+        <v>72</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="L11" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="M11" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="M11" s="1" t="s">
-        <v>194</v>
-      </c>
       <c r="N11" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="P11" s="1" t="s">
         <v>72</v>
@@ -4492,19 +4403,19 @@
         <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>193</v>
-      </c>
       <c r="E12" s="1" t="s">
-        <v>72</v>
+        <v>177</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>72</v>
@@ -4516,13 +4427,13 @@
         <v>72</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>197</v>
+        <v>72</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>72</v>
+        <v>183</v>
       </c>
       <c r="N12" s="1" t="s">
         <v>72</v>
@@ -4558,7 +4469,7 @@
         <v>8</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>72</v>
+        <v>182</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>72</v>
@@ -4567,7 +4478,7 @@
         <v>72</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>72</v>
@@ -4713,64 +4624,64 @@
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q18" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="I18" s="1" t="s">
+      <c r="S18" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K18" s="1" t="s">
+      <c r="T18" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="U18" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="V18" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="M18" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="N18" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="P18" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="S18" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="T18" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="U18" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="V18" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
@@ -4779,64 +4690,64 @@
         <v>2</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="S19" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I19" s="1" t="s">
+      <c r="T19" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="U19" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="O19" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="S19" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="T19" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="U19" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="V19" s="1" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
@@ -4845,64 +4756,64 @@
         <v>3</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>177</v>
+        <v>72</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="F20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q20" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G20" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="N20" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="O20" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="P20" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q20" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="R20" s="1" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="U20" s="1" t="s">
         <v>157</v>
       </c>
       <c r="V20" s="1" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
@@ -4923,52 +4834,52 @@
         <v>72</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>152</v>
+        <v>72</v>
       </c>
       <c r="H21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R21" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="I21" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="O21" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P21" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q21" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="R21" s="1" t="s">
-        <v>177</v>
-      </c>
       <c r="S21" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="T21" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="V21" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
@@ -5022,7 +4933,7 @@
         <v>72</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>177</v>
+        <v>72</v>
       </c>
       <c r="S22" s="1" t="s">
         <v>72</v>
@@ -5034,7 +4945,7 @@
         <v>72</v>
       </c>
       <c r="V22" s="1" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
@@ -5045,37 +4956,37 @@
         <v>6</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>193</v>
+        <v>72</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>72</v>
@@ -5117,31 +5028,31 @@
         <v>72</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J24" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="K24" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>72</v>
+        <v>183</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>197</v>
+        <v>176</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>72</v>
@@ -5332,64 +5243,64 @@
         <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="J30" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="K30" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="M30" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="N30" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="O30" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G30" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I30" s="1" t="s">
+      <c r="P30" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q30" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="R30" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="S30" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K30" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="L30" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="M30" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N30" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q30" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="R30" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="T30" s="1" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="U30" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="V30" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="V30" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
@@ -5398,64 +5309,64 @@
         <v>2</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="G31" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q31" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="R31" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H31" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="P31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q31" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="R31" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="S31" s="1" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="U31" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="V31" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="V31" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
@@ -5464,64 +5375,64 @@
         <v>3</v>
       </c>
       <c r="C32" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K32" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="L32" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="N32" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>154</v>
+        <v>72</v>
       </c>
       <c r="P32" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q32" s="1" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="R32" s="1" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="S32" s="1" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="T32" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="U32" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="U32" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="V32" s="1" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
@@ -5530,28 +5441,28 @@
         <v>4</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>195</v>
+        <v>72</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>181</v>
+        <v>72</v>
       </c>
       <c r="G33" s="1" t="s">
         <v>72</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>72</v>
+        <v>185</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>178</v>
+        <v>162</v>
       </c>
       <c r="K33" s="1" t="s">
         <v>72</v>
@@ -5560,34 +5471,34 @@
         <v>72</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="N33" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>154</v>
+        <v>72</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="S33" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="T33" s="1" t="s">
-        <v>72</v>
+        <v>156</v>
       </c>
       <c r="U33" s="1" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="V33" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
@@ -5617,7 +5528,7 @@
         <v>72</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>72</v>
@@ -5641,13 +5552,13 @@
         <v>72</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="T34" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="U34" s="1" t="s">
         <v>72</v>
@@ -5679,16 +5590,16 @@
         <v>72</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>184</v>
+        <v>72</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>199</v>
+        <v>72</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="L35" s="1" t="s">
         <v>72</v>
@@ -5697,10 +5608,10 @@
         <v>72</v>
       </c>
       <c r="N35" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="O35" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="P35" s="1" t="s">
         <v>72</v>
@@ -5763,10 +5674,10 @@
         <v>72</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="P36" s="1" t="s">
         <v>72</v>
@@ -5951,64 +5862,64 @@
         <v>1</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="M42" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="N42" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="O42" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="P42" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q42" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="R42" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H42" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="I42" s="1" t="s">
+      <c r="S42" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="J42" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="L42" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="M42" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N42" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="O42" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="P42" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q42" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="R42" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="S42" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="T42" s="1" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="U42" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="V42" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="V42" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
@@ -6017,64 +5928,64 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="J43" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="K43" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="M43" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="N43" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P43" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="R43" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="S43" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="T43" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="G43" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="L43" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="M43" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="N43" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="O43" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="P43" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q43" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="R43" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="S43" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T43" s="1" t="s">
+      <c r="U43" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="U43" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="V43" s="1" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
@@ -6083,64 +5994,64 @@
         <v>3</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="D44" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="M44" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="N44" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="O44" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P44" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q44" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="R44" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S44" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="T44" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="K44" s="1" t="s">
+      <c r="U44" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V44" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="L44" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="M44" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="N44" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O44" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P44" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q44" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="R44" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="S44" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="T44" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="U44" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="V44" s="1" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
@@ -6155,55 +6066,55 @@
         <v>72</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>181</v>
+        <v>72</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="G45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M45" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="H45" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="K45" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="L45" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M45" s="1" t="s">
+      <c r="N45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S45" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="T45" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="U45" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="N45" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P45" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q45" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="R45" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="S45" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="T45" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="U45" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="V45" s="1" t="s">
         <v>72</v>
@@ -6236,7 +6147,7 @@
         <v>72</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="K46" s="1" t="s">
         <v>72</v>
@@ -6269,7 +6180,7 @@
         <v>72</v>
       </c>
       <c r="U46" s="1" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
       <c r="V46" s="1" t="s">
         <v>72</v>
@@ -6292,16 +6203,16 @@
         <v>72</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>72</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>72</v>
+        <v>189</v>
       </c>
       <c r="J47" s="1" t="s">
         <v>72</v>
@@ -6310,16 +6221,16 @@
         <v>72</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="M47" s="1" t="s">
         <v>72</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="P47" s="1" t="s">
         <v>72</v>
@@ -6385,7 +6296,7 @@
         <v>72</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="P48" s="1" t="s">
         <v>72</v>
@@ -6570,64 +6481,64 @@
         <v>1</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="M54" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F54" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G54" s="1" t="s">
+      <c r="N54" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="O54" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q54" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="R54" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="S54" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="H54" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="L54" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="N54" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="O54" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="P54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q54" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="R54" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="S54" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="T54" s="1" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="U54" s="1" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="V54" s="1" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
@@ -6636,64 +6547,64 @@
         <v>2</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="H55" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J55" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="I55" s="1" t="s">
+      <c r="K55" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L55" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="M55" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="N55" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="O55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q55" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="J55" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="L55" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M55" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="N55" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="O55" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P55" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q55" s="1" t="s">
-        <v>176</v>
-      </c>
       <c r="R55" s="1" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="S55" s="1" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="T55" s="1" t="s">
-        <v>178</v>
+        <v>157</v>
       </c>
       <c r="U55" s="1" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="V55" s="1" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
@@ -6702,64 +6613,64 @@
         <v>3</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>196</v>
+        <v>146</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>72</v>
+        <v>143</v>
       </c>
       <c r="I56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K56" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="J56" s="1" t="s">
+      <c r="L56" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="M56" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="N56" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="O56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q56" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="R56" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="K56" s="1" t="s">
+      <c r="S56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T56" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U56" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="V56" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="L56" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="M56" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="N56" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="O56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q56" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="R56" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="S56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T56" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="U56" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="V56" s="1" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
@@ -6768,34 +6679,34 @@
         <v>4</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>195</v>
+        <v>164</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>72</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>72</v>
+        <v>170</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>72</v>
+        <v>143</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>72</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>72</v>
+        <v>162</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="M57" s="1" t="s">
         <v>72</v>
@@ -6810,22 +6721,22 @@
         <v>72</v>
       </c>
       <c r="Q57" s="1" t="s">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="R57" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="S57" s="1" t="s">
         <v>72</v>
       </c>
       <c r="T57" s="1" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="U57" s="1" t="s">
-        <v>72</v>
+        <v>156</v>
       </c>
       <c r="V57" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
@@ -6846,7 +6757,7 @@
         <v>72</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>72</v>
+        <v>162</v>
       </c>
       <c r="H58" s="1" t="s">
         <v>72</v>
@@ -6876,7 +6787,7 @@
         <v>72</v>
       </c>
       <c r="Q58" s="1" t="s">
-        <v>72</v>
+        <v>146</v>
       </c>
       <c r="R58" s="1" t="s">
         <v>72</v>
@@ -6885,7 +6796,7 @@
         <v>72</v>
       </c>
       <c r="T58" s="1" t="s">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="U58" s="1" t="s">
         <v>72</v>
@@ -6926,13 +6837,13 @@
         <v>72</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="L59" s="1" t="s">
         <v>72</v>
       </c>
       <c r="M59" s="1" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="N59" s="1" t="s">
         <v>72</v>
@@ -7189,64 +7100,64 @@
         <v>1</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="F66" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="M66" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="N66" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="O66" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P66" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q66" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="R66" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="S66" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="T66" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="U66" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="V66" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="I66" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="J66" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="L66" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M66" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="N66" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="O66" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="P66" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q66" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="R66" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="S66" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="T66" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="U66" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="V66" s="1" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
@@ -7255,64 +7166,64 @@
         <v>2</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F67" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="L67" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="L67" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="M67" s="1" t="s">
         <v>160</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>171</v>
+        <v>145</v>
       </c>
       <c r="O67" s="1" t="s">
-        <v>72</v>
+        <v>151</v>
       </c>
       <c r="P67" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q67" s="1" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="R67" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="S67" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="T67" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="U67" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="S67" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="T67" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="U67" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="V67" s="1" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
@@ -7321,64 +7232,64 @@
         <v>3</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="D68" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="J68" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="E68" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I68" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="K68" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>161</v>
+        <v>72</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>72</v>
+        <v>151</v>
       </c>
       <c r="P68" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q68" s="1" t="s">
-        <v>174</v>
+        <v>152</v>
       </c>
       <c r="R68" s="1" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="S68" s="1" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="T68" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U68" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="V68" s="1" t="s">
-        <v>165</v>
+        <v>72</v>
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
@@ -7390,16 +7301,16 @@
         <v>72</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>173</v>
+        <v>72</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>72</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>181</v>
+        <v>72</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="H69" s="1" t="s">
         <v>72</v>
@@ -7408,7 +7319,7 @@
         <v>72</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>72</v>
+        <v>162</v>
       </c>
       <c r="K69" s="1" t="s">
         <v>72</v>
@@ -7420,10 +7331,10 @@
         <v>72</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>179</v>
+        <v>150</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="P69" s="1" t="s">
         <v>72</v>
@@ -7432,7 +7343,7 @@
         <v>72</v>
       </c>
       <c r="R69" s="1" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="S69" s="1" t="s">
         <v>72</v>
@@ -7441,10 +7352,10 @@
         <v>72</v>
       </c>
       <c r="U69" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="V69" s="1" t="s">
-        <v>167</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
@@ -7548,13 +7459,13 @@
         <v>72</v>
       </c>
       <c r="L71" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="M71" s="1" t="s">
         <v>72</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="O71" s="1" t="s">
         <v>72</v>

</xml_diff>